<commit_message>
working on risk management
</commit_message>
<xml_diff>
--- a/content/tables/Risk_Mgmt.xlsx
+++ b/content/tables/Risk_Mgmt.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BFH\MSE\MSE_MasterThesis\content\tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E478648B-2632-4823-AC65-1E8805AA94FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBDF98A1-9C73-4045-98A2-EEEDBA3AC342}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{C85C79CF-50DE-474C-BA2B-673335091AFF}"/>
   </bookViews>
   <sheets>
     <sheet name="Table with Risks and Measures" sheetId="5" r:id="rId1"/>
-    <sheet name="Graphical Overview" sheetId="4" r:id="rId2"/>
-    <sheet name="RiskEval" sheetId="6" r:id="rId3"/>
-    <sheet name="RiskTreatment" sheetId="7" r:id="rId4"/>
-    <sheet name="RiskWhatWhen" sheetId="8" r:id="rId5"/>
-    <sheet name="CheckinOct" sheetId="12" r:id="rId6"/>
+    <sheet name="Table with Risks_Projekt2" sheetId="13" r:id="rId2"/>
+    <sheet name="Graphical Overview" sheetId="4" r:id="rId3"/>
+    <sheet name="RiskEval" sheetId="6" r:id="rId4"/>
+    <sheet name="RiskTreatment" sheetId="7" r:id="rId5"/>
+    <sheet name="RiskWhatWhen" sheetId="8" r:id="rId6"/>
+    <sheet name="CheckinOct" sheetId="12" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Graphical Overview'!$J$1:$L$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Table with Risks and Measures'!$E$1:$E$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Graphical Overview'!$J$1:$L$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Table with Risks and Measures'!$E$1:$E$33</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="169">
   <si>
     <t>Risk</t>
   </si>
@@ -296,9 +297,6 @@
     <t>To be documented in miro calendar case it happens</t>
   </si>
   <si>
-    <t>4, 6, 10, 12</t>
-  </si>
-  <si>
     <t>Treatment</t>
   </si>
   <si>
@@ -476,9 +474,6 @@
     <t>Insufficient scientific contribution</t>
   </si>
   <si>
-    <t>This research does not add new research to the initiative</t>
-  </si>
-  <si>
     <t>Learning is part of the journey but additional time is to planed</t>
   </si>
   <si>
@@ -488,21 +483,6 @@
     <t>Happened before start, Provide contact of partner working at BFH, Document in case it hapens</t>
   </si>
   <si>
-    <t>3, 22</t>
-  </si>
-  <si>
-    <t>9, 21</t>
-  </si>
-  <si>
-    <t>17, 23</t>
-  </si>
-  <si>
-    <t>11, 13, 15, 19</t>
-  </si>
-  <si>
-    <t>14, 16, 18, 20</t>
-  </si>
-  <si>
     <t>Providing continous feedback and having weekly call are done to find missing contributions early</t>
   </si>
   <si>
@@ -525,6 +505,54 @@
   </si>
   <si>
     <t>Accept: Exchange with teams</t>
+  </si>
+  <si>
+    <t>4, 12</t>
+  </si>
+  <si>
+    <t>6, 10</t>
+  </si>
+  <si>
+    <t>Provide contact of partner working at BFH, Document in case it hapens</t>
+  </si>
+  <si>
+    <t>Risk is accepted, learning is wanted effect</t>
+  </si>
+  <si>
+    <t>Checkup Action or OK</t>
+  </si>
+  <si>
+    <t>Checkup When</t>
+  </si>
+  <si>
+    <t>Project 1 and 2 established much of the required steps, however it is still likely that something new can pop up</t>
+  </si>
+  <si>
+    <t>Reduce: Still important to handle them as soon as they apear</t>
+  </si>
+  <si>
+    <t>13, 15, 19, 23</t>
+  </si>
+  <si>
+    <t>14, 18</t>
+  </si>
+  <si>
+    <t>5, 9</t>
+  </si>
+  <si>
+    <t>21, 22</t>
+  </si>
+  <si>
+    <t>3, 20</t>
+  </si>
+  <si>
+    <t>This research does not add sufficient scientific value</t>
+  </si>
+  <si>
+    <t>The resopnsible parties need to be found first</t>
+  </si>
+  <si>
+    <t>The required management process is unknown</t>
   </si>
 </sst>
 </file>
@@ -562,7 +590,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -611,6 +639,24 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -650,7 +696,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
@@ -671,18 +717,33 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1017,7 +1078,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01ACE7B3-DC9E-49CA-A001-535C01F14776}">
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:X33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.89453125" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="10.89453125" style="2"/>
@@ -1027,13 +1088,13 @@
     <col min="5" max="5" width="9.1015625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.734375" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="20.26171875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="11" width="10.89453125" style="1"/>
-    <col min="12" max="12" width="51.47265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.15625" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="10.89453125" style="1"/>
+    <col min="8" max="21" width="10.89453125" style="1"/>
+    <col min="22" max="22" width="51.47265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="14.15625" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="16384" width="10.89453125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="23.7" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:24" ht="23.7" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="3" t="s">
         <v>55</v>
       </c>
@@ -1055,29 +1116,53 @@
       <c r="G1" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="M1" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="N1" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="O1" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="P1" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q1" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="R1" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="S1" s="3"/>
+      <c r="T1" s="3"/>
+      <c r="U1" s="3"/>
+      <c r="V1" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="N1" s="1" t="s">
+      <c r="W1" s="3" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="X1" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -1103,17 +1188,33 @@
       <c r="I2" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="L2" s="22">
+        <v>2</v>
+      </c>
+      <c r="M2" s="20">
+        <v>2</v>
+      </c>
+      <c r="N2" s="20">
+        <f>L2*M2</f>
+        <v>4</v>
+      </c>
+      <c r="O2" s="21"/>
+      <c r="P2" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q2" s="21"/>
+      <c r="R2" s="21"/>
+      <c r="V2" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="M2" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="N2" s="7">
+      <c r="W2" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="X2" s="7">
         <v>46319</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -1133,23 +1234,39 @@
         <v>3</v>
       </c>
       <c r="G3" s="6">
-        <f t="shared" ref="G3:G26" si="0">E3*F3</f>
+        <f t="shared" ref="G3:G23" si="0">E3*F3</f>
         <v>6</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="L3" s="22">
+        <v>2</v>
+      </c>
+      <c r="M3" s="20">
+        <v>3</v>
+      </c>
+      <c r="N3" s="20">
+        <f>L3*M3</f>
+        <v>6</v>
+      </c>
+      <c r="O3" s="21"/>
+      <c r="P3" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q3" s="21"/>
+      <c r="R3" s="21"/>
+      <c r="V3" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="M3" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="N3" s="7">
+      <c r="W3" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="X3" s="7">
         <v>46319</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -1175,53 +1292,82 @@
       <c r="I4" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="L4" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="N4" s="7">
+      <c r="L4" s="22">
+        <v>4</v>
+      </c>
+      <c r="M4" s="20">
+        <v>2</v>
+      </c>
+      <c r="N4" s="20">
+        <f>L4*M4</f>
+        <v>8</v>
+      </c>
+      <c r="O4" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="P4" s="21"/>
+      <c r="Q4" s="21"/>
+      <c r="R4" s="21"/>
+      <c r="V4" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="W4" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="X4" s="7">
         <v>46319</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="3">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3" t="s">
+    <row r="5" spans="1:24" s="25" customFormat="1" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="23">
+        <v>4</v>
+      </c>
+      <c r="B5" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="5">
-        <v>4</v>
-      </c>
-      <c r="F5" s="6">
-        <v>3</v>
-      </c>
-      <c r="G5" s="6">
+      <c r="E5" s="24">
+        <v>4</v>
+      </c>
+      <c r="F5" s="23">
+        <v>4</v>
+      </c>
+      <c r="G5" s="23">
         <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="I5" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="L5" s="24">
+        <v>4</v>
+      </c>
+      <c r="M5" s="23">
+        <v>3</v>
+      </c>
+      <c r="N5" s="23">
+        <f>L5*M5</f>
         <v>12</v>
       </c>
-      <c r="I5" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="N5" s="7">
+      <c r="O5" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="V5" s="25" t="s">
+        <v>143</v>
+      </c>
+      <c r="W5" s="25" t="s">
+        <v>90</v>
+      </c>
+      <c r="X5" s="26">
         <v>46319</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -1247,17 +1393,33 @@
       <c r="H6" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="L6" s="22">
+        <v>3</v>
+      </c>
+      <c r="M6" s="20">
+        <v>3</v>
+      </c>
+      <c r="N6" s="20">
+        <f>L6*M6</f>
+        <v>9</v>
+      </c>
+      <c r="O6" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="P6" s="21"/>
+      <c r="Q6" s="21"/>
+      <c r="R6" s="21"/>
+      <c r="V6" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="M6" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="N6" s="7">
+      <c r="W6" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="X6" s="7">
         <v>46319</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:24" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -1283,17 +1445,33 @@
       <c r="I7" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="L7" s="1" t="s">
+      <c r="L7" s="22">
+        <v>4</v>
+      </c>
+      <c r="M7" s="20">
+        <v>3</v>
+      </c>
+      <c r="N7" s="20">
+        <f>L7*M7</f>
+        <v>12</v>
+      </c>
+      <c r="O7" s="21"/>
+      <c r="P7" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q7" s="21"/>
+      <c r="R7" s="21"/>
+      <c r="V7" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="M7" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="N7" s="7">
+      <c r="W7" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="X7" s="7">
         <v>46319</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -1319,89 +1497,131 @@
       <c r="I8" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="L8" s="1" t="s">
+      <c r="L8" s="22">
+        <v>3</v>
+      </c>
+      <c r="M8" s="20">
+        <v>2</v>
+      </c>
+      <c r="N8" s="20">
+        <f>L8*M8</f>
+        <v>6</v>
+      </c>
+      <c r="O8" s="21"/>
+      <c r="P8" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q8" s="21"/>
+      <c r="R8" s="21"/>
+      <c r="V8" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="M8" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="N8" s="7">
+      <c r="W8" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="X8" s="7">
         <v>46319</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="3">
+    <row r="9" spans="1:24" s="25" customFormat="1" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="23">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="E9" s="5">
-        <v>5</v>
-      </c>
-      <c r="F9" s="6">
-        <v>4</v>
-      </c>
-      <c r="G9" s="6">
+      <c r="E9" s="24">
+        <v>5</v>
+      </c>
+      <c r="F9" s="23">
+        <v>4</v>
+      </c>
+      <c r="G9" s="23">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="I9" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="L9" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="M9" s="1" t="s">
+      <c r="I9" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="L9" s="24">
+        <v>4</v>
+      </c>
+      <c r="M9" s="23">
+        <v>4</v>
+      </c>
+      <c r="N9" s="23">
+        <f>L9*M9</f>
+        <v>16</v>
+      </c>
+      <c r="P9" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="V9" s="25" t="s">
+        <v>144</v>
+      </c>
+      <c r="W9" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="X9" s="26">
+        <v>46319</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" s="25" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="23">
+        <v>9</v>
+      </c>
+      <c r="B10" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="E10" s="27">
+        <v>3</v>
+      </c>
+      <c r="F10" s="28">
+        <v>3</v>
+      </c>
+      <c r="G10" s="28">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="J10" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="L10" s="24">
+        <v>3</v>
+      </c>
+      <c r="M10" s="23">
+        <v>4</v>
+      </c>
+      <c r="N10" s="23">
+        <f>L10*M10</f>
+        <v>12</v>
+      </c>
+      <c r="Q10" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="V10" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="W10" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="N9" s="7">
+      <c r="X10" s="26">
         <v>46319</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="3">
-        <v>9</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="E10" s="5">
-        <v>3</v>
-      </c>
-      <c r="F10" s="6">
-        <v>4</v>
-      </c>
-      <c r="G10" s="6">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="L10" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="M10" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="N10" s="7">
-        <v>46319</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -1427,485 +1647,646 @@
       <c r="H11" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="L11" s="1" t="s">
+      <c r="L11" s="22">
+        <v>4</v>
+      </c>
+      <c r="M11" s="20">
+        <v>3</v>
+      </c>
+      <c r="N11" s="20">
+        <f>L11*M11</f>
+        <v>12</v>
+      </c>
+      <c r="O11" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="P11" s="21"/>
+      <c r="Q11" s="21"/>
+      <c r="R11" s="21"/>
+      <c r="V11" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="M11" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="N11" s="7">
+      <c r="W11" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="X11" s="7">
         <v>46319</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="3">
+    <row r="12" spans="1:24" s="25" customFormat="1" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="23">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="E12" s="5">
-        <v>2</v>
-      </c>
-      <c r="F12" s="6">
-        <v>5</v>
-      </c>
-      <c r="G12" s="6">
+      <c r="E12" s="24">
+        <v>2</v>
+      </c>
+      <c r="F12" s="23">
+        <v>4</v>
+      </c>
+      <c r="G12" s="23">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="I12" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="L12" s="24">
+        <v>2</v>
+      </c>
+      <c r="M12" s="23">
+        <v>5</v>
+      </c>
+      <c r="N12" s="23">
+        <f>L12*M12</f>
+        <v>10</v>
+      </c>
+      <c r="P12" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="V12" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="W12" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="X12" s="26">
+        <v>46319</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" s="25" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="23">
+        <v>12</v>
+      </c>
+      <c r="B13" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" s="24">
+        <v>4</v>
+      </c>
+      <c r="F13" s="23">
+        <v>4</v>
+      </c>
+      <c r="G13" s="23">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="H13" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="L13" s="24">
+        <v>4</v>
+      </c>
+      <c r="M13" s="23">
+        <v>3</v>
+      </c>
+      <c r="N13" s="23">
+        <f>L13*M13</f>
+        <v>12</v>
+      </c>
+      <c r="O13" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="V13" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="W13" s="25" t="s">
+        <v>90</v>
+      </c>
+      <c r="X13" s="26">
+        <v>46319</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" s="25" customFormat="1" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="23">
+        <v>13</v>
+      </c>
+      <c r="B14" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E14" s="27">
+        <v>1</v>
+      </c>
+      <c r="F14" s="28">
+        <v>5</v>
+      </c>
+      <c r="G14" s="28">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="I14" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="L14" s="24">
+        <v>2</v>
+      </c>
+      <c r="M14" s="23">
+        <v>5</v>
+      </c>
+      <c r="N14" s="23">
+        <f>L14*M14</f>
+        <v>10</v>
+      </c>
+      <c r="P14" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="V14" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="W14" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="X14" s="26">
+        <v>46319</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="3">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E15" s="5">
+        <v>2</v>
+      </c>
+      <c r="F15" s="6">
+        <v>5</v>
+      </c>
+      <c r="G15" s="6">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="I12" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="L12" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="M12" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="N12" s="7">
+      <c r="I15" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="L15" s="22">
+        <v>2</v>
+      </c>
+      <c r="M15" s="20">
+        <v>5</v>
+      </c>
+      <c r="N15" s="20">
+        <f>L15*M15</f>
+        <v>10</v>
+      </c>
+      <c r="O15" s="21"/>
+      <c r="P15" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q15" s="21"/>
+      <c r="R15" s="21"/>
+      <c r="V15" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="W15" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="X15" s="7">
         <v>46319</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="3">
+    <row r="16" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" s="3">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" s="5">
+        <v>1</v>
+      </c>
+      <c r="F16" s="6">
+        <v>5</v>
+      </c>
+      <c r="G16" s="6">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="L16" s="22">
+        <v>1</v>
+      </c>
+      <c r="M16" s="20">
+        <v>5</v>
+      </c>
+      <c r="N16" s="20">
+        <f>L16*M16</f>
+        <v>5</v>
+      </c>
+      <c r="O16" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="P16" s="21"/>
+      <c r="Q16" s="21"/>
+      <c r="R16" s="21"/>
+      <c r="V16" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="W16" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="X16" s="7">
+        <v>46319</v>
+      </c>
+    </row>
+    <row r="17" spans="1:24" s="25" customFormat="1" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17" s="23">
+        <v>16</v>
+      </c>
+      <c r="B17" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="E17" s="27">
+        <v>1</v>
+      </c>
+      <c r="F17" s="28">
+        <v>4</v>
+      </c>
+      <c r="G17" s="28">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="I17" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="L17" s="24">
+        <v>2</v>
+      </c>
+      <c r="M17" s="23">
+        <v>4</v>
+      </c>
+      <c r="N17" s="23">
+        <f>L17*M17</f>
+        <v>8</v>
+      </c>
+      <c r="P17" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="V17" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="W17" s="25" t="s">
+        <v>103</v>
+      </c>
+      <c r="X17" s="26">
+        <v>46319</v>
+      </c>
+    </row>
+    <row r="18" spans="1:24" s="25" customFormat="1" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" s="23">
+        <v>17</v>
+      </c>
+      <c r="B18" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="C18" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="D18" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="E18" s="24">
+        <v>3</v>
+      </c>
+      <c r="F18" s="23">
+        <v>5</v>
+      </c>
+      <c r="G18" s="23">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="I18" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="L18" s="24">
+        <v>1</v>
+      </c>
+      <c r="M18" s="23">
+        <v>5</v>
+      </c>
+      <c r="N18" s="23">
+        <f>L18*M18</f>
+        <v>5</v>
+      </c>
+      <c r="P18" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="V18" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="W18" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="X18" s="26">
+        <v>46319</v>
+      </c>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19" s="3">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19" s="5">
+        <v>2</v>
+      </c>
+      <c r="F19" s="6">
+        <v>5</v>
+      </c>
+      <c r="G19" s="6">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="L19" s="22">
+        <v>2</v>
+      </c>
+      <c r="M19" s="20">
+        <v>5</v>
+      </c>
+      <c r="N19" s="20">
+        <f>L19*M19</f>
+        <v>10</v>
+      </c>
+      <c r="O19" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="P19" s="21"/>
+      <c r="Q19" s="21"/>
+      <c r="R19" s="21"/>
+      <c r="V19" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="W19" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="X19" s="7">
+        <v>46319</v>
+      </c>
+    </row>
+    <row r="20" spans="1:24" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A20" s="3">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="E20" s="5">
+        <v>1</v>
+      </c>
+      <c r="F20" s="6">
+        <v>5</v>
+      </c>
+      <c r="G20" s="6">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="L20" s="22">
+        <v>1</v>
+      </c>
+      <c r="M20" s="20">
+        <v>5</v>
+      </c>
+      <c r="N20" s="20">
+        <f>L20*M20</f>
+        <v>5</v>
+      </c>
+      <c r="O20" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="P20" s="21"/>
+      <c r="Q20" s="21"/>
+      <c r="R20" s="21"/>
+      <c r="V20" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="W20" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="X20" s="7">
+        <v>46319</v>
+      </c>
+    </row>
+    <row r="21" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A21" s="3">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="E21" s="27">
+        <v>4</v>
+      </c>
+      <c r="F21" s="28">
+        <v>2</v>
+      </c>
+      <c r="G21" s="28">
+        <f>E21*F21</f>
+        <v>8</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="L21" s="22">
+        <v>5</v>
+      </c>
+      <c r="M21" s="20">
+        <v>3</v>
+      </c>
+      <c r="N21" s="20">
+        <f>L21*M21</f>
+        <v>15</v>
+      </c>
+      <c r="O21" s="21"/>
+      <c r="P21" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q21" s="21"/>
+      <c r="R21" s="21"/>
+      <c r="V21" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="W21" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="X21" s="7">
+        <v>46319</v>
+      </c>
+    </row>
+    <row r="22" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A22" s="3">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="E22" s="5">
+        <v>3</v>
+      </c>
+      <c r="F22" s="6">
+        <v>4</v>
+      </c>
+      <c r="G22" s="6">
+        <f>E22*F22</f>
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="E13" s="5">
-        <v>4</v>
-      </c>
-      <c r="F13" s="6">
-        <v>3</v>
-      </c>
-      <c r="G13" s="6">
+      <c r="I22" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="V22" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="W22" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="X22" s="7">
+        <v>46319</v>
+      </c>
+    </row>
+    <row r="23" spans="1:24" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A23" s="3">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="E23" s="5">
+        <v>3</v>
+      </c>
+      <c r="F23" s="6">
+        <v>4</v>
+      </c>
+      <c r="G23" s="6">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="H13" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="L13" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="M13" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="N13" s="7">
+      <c r="H23" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="V23" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="W23" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="X23" s="7">
         <v>46319</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="3">
-        <v>13</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="E14" s="5">
-        <v>2</v>
-      </c>
-      <c r="F14" s="6">
-        <v>5</v>
-      </c>
-      <c r="G14" s="6">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="L14" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="M14" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="N14" s="7">
-        <v>46319</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A15" s="3">
-        <v>14</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="E15" s="5">
-        <v>1</v>
-      </c>
-      <c r="F15" s="6">
-        <v>5</v>
-      </c>
-      <c r="G15" s="6">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="L15" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="M15" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="N15" s="7">
-        <v>46319</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="3">
-        <v>15</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="E16" s="5">
-        <v>2</v>
-      </c>
-      <c r="F16" s="6">
-        <v>5</v>
-      </c>
-      <c r="G16" s="6">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="L16" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="M16" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="N16" s="7">
-        <v>46319</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A17" s="3">
-        <v>16</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="E17" s="5">
-        <v>1</v>
-      </c>
-      <c r="F17" s="6">
-        <v>5</v>
-      </c>
-      <c r="G17" s="6">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="L17" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="M17" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="N17" s="7">
-        <v>46319</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" s="3">
-        <v>17</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="E18" s="5">
-        <v>2</v>
-      </c>
-      <c r="F18" s="6">
-        <v>4</v>
-      </c>
-      <c r="G18" s="6">
-        <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="L18" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="M18" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="N18" s="7">
-        <v>46319</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="3">
-        <v>18</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E19" s="5">
-        <v>1</v>
-      </c>
-      <c r="F19" s="6">
-        <v>5</v>
-      </c>
-      <c r="G19" s="6">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="L19" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="M19" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="N19" s="7">
-        <v>46319</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.55000000000000004">
-      <c r="A20" s="3">
-        <v>19</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="E20" s="5">
-        <v>2</v>
-      </c>
-      <c r="F20" s="6">
-        <v>5</v>
-      </c>
-      <c r="G20" s="6">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="L20" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="M20" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="N20" s="7">
-        <v>46319</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A21" s="3">
-        <v>20</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="E21" s="5">
-        <v>1</v>
-      </c>
-      <c r="F21" s="6">
-        <v>5</v>
-      </c>
-      <c r="G21" s="6">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="L21" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="M21" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="N21" s="7">
-        <v>46319</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="3">
-        <v>21</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="E22" s="5">
-        <v>3</v>
-      </c>
-      <c r="F22" s="6">
-        <v>4</v>
-      </c>
-      <c r="G22" s="6">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="I22" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="L22" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M22" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="N22" s="7">
-        <v>46319</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A23" s="3">
-        <v>22</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="E23" s="5">
-        <v>4</v>
-      </c>
-      <c r="F23" s="6">
-        <v>2</v>
-      </c>
-      <c r="G23" s="6">
-        <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="L23" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="M23" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="N23" s="7">
-        <v>46319</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="3">
         <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>135</v>
+        <v>37</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>141</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>140</v>
+        <v>166</v>
       </c>
       <c r="E24" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F24" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G24" s="6">
-        <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="L24" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="M24" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="N24" s="7">
+        <f>E24*F24</f>
+        <v>5</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="V24" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="W24" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="X24" s="7">
         <v>46319</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="5"/>
@@ -1913,9 +2294,9 @@
       <c r="E25" s="5"/>
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
-      <c r="N25" s="7"/>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="X25" s="7"/>
+    </row>
+    <row r="26" spans="1:24" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="5"/>
@@ -1923,19 +2304,19 @@
       <c r="E26" s="5"/>
       <c r="F26" s="6"/>
       <c r="G26" s="6"/>
-      <c r="N26" s="7"/>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="X26" s="7"/>
+    </row>
+    <row r="27" spans="1:24" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
-      <c r="C27" s="5"/>
+      <c r="C27"/>
       <c r="D27" s="5"/>
       <c r="E27" s="5"/>
       <c r="F27" s="6"/>
       <c r="G27" s="6"/>
-      <c r="N27" s="7"/>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="X27" s="7"/>
+    </row>
+    <row r="28" spans="1:24" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28"/>
@@ -1943,66 +2324,860 @@
       <c r="E28" s="5"/>
       <c r="F28" s="6"/>
       <c r="G28" s="6"/>
-      <c r="N28" s="7"/>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
+      <c r="X28" s="7"/>
+    </row>
+    <row r="29" spans="1:24" x14ac:dyDescent="0.55000000000000004">
       <c r="C29"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="6"/>
-      <c r="G29" s="6"/>
-      <c r="N29" s="7"/>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="30" spans="1:24" x14ac:dyDescent="0.55000000000000004">
       <c r="C30"/>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="1:24" x14ac:dyDescent="0.55000000000000004">
       <c r="C31"/>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="1:24" x14ac:dyDescent="0.55000000000000004">
       <c r="C32"/>
     </row>
     <row r="33" spans="3:3" x14ac:dyDescent="0.55000000000000004">
       <c r="C33"/>
     </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="C34"/>
-    </row>
   </sheetData>
-  <autoFilter ref="E1:E34" xr:uid="{01ACE7B3-DC9E-49CA-A001-535C01F14776}"/>
+  <autoFilter ref="E1:E33" xr:uid="{01ACE7B3-DC9E-49CA-A001-535C01F14776}"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2E3A70C-6FBC-4F85-BBC7-0384E51FABE2}">
+  <dimension ref="A1:AM21"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.89453125" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="10.89453125" style="2"/>
+    <col min="2" max="2" width="18.1015625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="52.5234375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.5234375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.1015625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.26171875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="20" width="10.89453125" style="1"/>
+    <col min="21" max="21" width="51.47265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.15625" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="16384" width="10.89453125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:25" ht="23.7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="5">
+        <v>2</v>
+      </c>
+      <c r="F2" s="6">
+        <v>2</v>
+      </c>
+      <c r="G2" s="6">
+        <f>E2*F2</f>
+        <v>4</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="W2" s="7">
+        <v>72981</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="5">
+        <v>2</v>
+      </c>
+      <c r="F3" s="6">
+        <v>3</v>
+      </c>
+      <c r="G3" s="6">
+        <f>E3*F3</f>
+        <v>6</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U3" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="V3" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E4" s="5">
+        <v>4</v>
+      </c>
+      <c r="F4" s="6">
+        <v>2</v>
+      </c>
+      <c r="G4" s="6">
+        <f>E4*F4</f>
+        <v>8</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U4" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="V4" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="W4" s="7">
+        <v>45953</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="5">
+        <v>4</v>
+      </c>
+      <c r="F5" s="6">
+        <v>3</v>
+      </c>
+      <c r="G5" s="6">
+        <f>E5*F5</f>
+        <v>12</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U5" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="V5" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="W5" s="7">
+        <v>45953</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="5">
+        <v>3</v>
+      </c>
+      <c r="F6" s="6">
+        <v>3</v>
+      </c>
+      <c r="G6" s="6">
+        <f>E6*F6</f>
+        <v>9</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U6" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="V6" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="W6" s="7">
+        <v>45953</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="E7" s="5">
+        <v>4</v>
+      </c>
+      <c r="F7" s="6">
+        <v>3</v>
+      </c>
+      <c r="G7" s="6">
+        <f>E7*F7</f>
+        <v>12</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U7" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="V7" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="W7" s="7">
+        <v>45940</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="5">
+        <v>3</v>
+      </c>
+      <c r="F8" s="6">
+        <v>2</v>
+      </c>
+      <c r="G8" s="6">
+        <f>E8*F8</f>
+        <v>6</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U8" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="V8" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="W8" s="7">
+        <v>45947</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" s="5">
+        <v>4</v>
+      </c>
+      <c r="F9" s="6">
+        <v>4</v>
+      </c>
+      <c r="G9" s="6">
+        <f>E9*F9</f>
+        <v>16</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U9" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="V9" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="W9" s="7">
+        <v>45953</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E10" s="5">
+        <v>3</v>
+      </c>
+      <c r="F10" s="6">
+        <v>4</v>
+      </c>
+      <c r="G10" s="6">
+        <f>E10*F10</f>
+        <v>12</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U10" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="V10" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="W10" s="7">
+        <v>45953</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="5">
+        <v>4</v>
+      </c>
+      <c r="F11" s="6">
+        <v>3</v>
+      </c>
+      <c r="G11" s="6">
+        <f>E11*F11</f>
+        <v>12</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U11" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="V11" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="W11" s="7">
+        <v>45953</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="3">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12" s="5">
+        <v>2</v>
+      </c>
+      <c r="F12" s="6">
+        <v>5</v>
+      </c>
+      <c r="G12" s="6">
+        <f>E12*F12</f>
+        <v>10</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U12" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="V12" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="W12" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="13" spans="1:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="3">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" s="5">
+        <v>4</v>
+      </c>
+      <c r="F13" s="6">
+        <v>3</v>
+      </c>
+      <c r="G13" s="6">
+        <f>E13*F13</f>
+        <v>12</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U13" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="V13" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="W13" s="7">
+        <v>45953</v>
+      </c>
+    </row>
+    <row r="14" spans="1:25" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="3">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E14" s="5">
+        <v>2</v>
+      </c>
+      <c r="F14" s="6">
+        <v>5</v>
+      </c>
+      <c r="G14" s="6">
+        <f>E14*F14</f>
+        <v>10</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U14" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="V14" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="W14" s="7">
+        <v>45940</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="3">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E15" s="5">
+        <v>2</v>
+      </c>
+      <c r="F15" s="6">
+        <v>5</v>
+      </c>
+      <c r="G15" s="6">
+        <f>E15*F15</f>
+        <v>10</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U15" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="V15" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="W15" s="7">
+        <v>45947</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" s="3">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" s="5">
+        <v>1</v>
+      </c>
+      <c r="F16" s="6">
+        <v>5</v>
+      </c>
+      <c r="G16" s="6">
+        <f>E16*F16</f>
+        <v>5</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U16" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="V16" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="W16" s="7">
+        <v>45940</v>
+      </c>
+    </row>
+    <row r="17" spans="1:39" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17" s="3">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E17" s="5">
+        <v>2</v>
+      </c>
+      <c r="F17" s="6">
+        <v>4</v>
+      </c>
+      <c r="G17" s="6">
+        <f>E17*F17</f>
+        <v>8</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U17" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="V17" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="W17" s="7">
+        <v>45926</v>
+      </c>
+    </row>
+    <row r="18" spans="1:39" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" s="3">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E18" s="5">
+        <v>1</v>
+      </c>
+      <c r="F18" s="6">
+        <v>5</v>
+      </c>
+      <c r="G18" s="6">
+        <f>E18*F18</f>
+        <v>5</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U18" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="V18" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="W18" s="7">
+        <v>45926</v>
+      </c>
+    </row>
+    <row r="19" spans="1:39" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19" s="3">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19" s="5">
+        <v>2</v>
+      </c>
+      <c r="F19" s="6">
+        <v>5</v>
+      </c>
+      <c r="G19" s="6">
+        <f>E19*F19</f>
+        <v>10</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U19" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="V19" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="W19" s="7">
+        <v>45953</v>
+      </c>
+    </row>
+    <row r="20" spans="1:39" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A20" s="3">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="E20" s="5">
+        <v>1</v>
+      </c>
+      <c r="F20" s="6">
+        <v>5</v>
+      </c>
+      <c r="G20" s="6">
+        <f>E20*F20</f>
+        <v>5</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="U20" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="V20" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="W20" s="7">
+        <v>45953</v>
+      </c>
+    </row>
+    <row r="21" spans="1:39" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A21" s="3">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="E21" s="5">
+        <v>5</v>
+      </c>
+      <c r="F21" s="6">
+        <v>3</v>
+      </c>
+      <c r="G21" s="6">
+        <f>E21*F21</f>
+        <v>15</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="AK21" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="AL21" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="AM21" s="7">
+        <v>46319</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38F3AE2C-2824-4C08-B947-28E1493E0DC2}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="B2:L37"/>
+  <dimension ref="B1:R37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="3" max="3" width="12.15625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.89453125" style="2"/>
+    <col min="11" max="11" width="9.1015625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.26171875" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.89453125" style="2"/>
+    <col min="15" max="15" width="9.1015625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="6.734375" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B2" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-    </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B3" s="13"/>
-      <c r="C3" s="14"/>
+    <row r="1" spans="2:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="N1" s="3"/>
+      <c r="O1" s="3"/>
+      <c r="P1" s="3"/>
+    </row>
+    <row r="2" spans="2:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="B2" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="5"/>
+      <c r="P2" s="6"/>
+    </row>
+    <row r="3" spans="2:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="B3" s="19"/>
+      <c r="C3" s="13"/>
       <c r="D3" s="3" t="s">
         <v>10</v>
       </c>
@@ -2018,85 +3193,134 @@
       <c r="H3" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="2:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B4" s="13"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="6"/>
+    </row>
+    <row r="4" spans="2:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B4" s="19"/>
       <c r="C4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="16"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18">
+      <c r="D4" s="14"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16">
         <v>8</v>
       </c>
-      <c r="H4" s="18"/>
-    </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B5" s="13"/>
+      <c r="H4" s="16"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="5"/>
+      <c r="P4" s="6"/>
+    </row>
+    <row r="5" spans="2:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="B5" s="19"/>
       <c r="C5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="16"/>
-      <c r="E5" s="17" t="s">
-        <v>147</v>
-      </c>
-      <c r="F5" s="17" t="s">
-        <v>83</v>
-      </c>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-    </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="13"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>153</v>
+      </c>
+      <c r="H5" s="16"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="5"/>
+      <c r="P5" s="6"/>
+    </row>
+    <row r="6" spans="2:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="B6" s="19"/>
       <c r="C6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="19"/>
-      <c r="E6" s="16">
+      <c r="D6" s="17"/>
+      <c r="E6" s="14">
         <v>7</v>
       </c>
-      <c r="F6" s="17">
-        <v>5</v>
-      </c>
-      <c r="G6" s="17" t="s">
-        <v>148</v>
-      </c>
-      <c r="H6" s="18"/>
-    </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B7" s="13"/>
+      <c r="F6" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="G6" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="H6" s="16">
+        <v>17</v>
+      </c>
+      <c r="N6" s="3"/>
+      <c r="O6" s="5"/>
+      <c r="P6" s="6"/>
+    </row>
+    <row r="7" spans="2:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="B7" s="19"/>
       <c r="C7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19">
+      <c r="D7" s="17"/>
+      <c r="E7" s="17">
         <v>1</v>
       </c>
-      <c r="F7" s="16">
-        <v>2</v>
-      </c>
-      <c r="G7" s="16" t="s">
-        <v>149</v>
-      </c>
-      <c r="H7" s="17" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="B8" s="13"/>
+      <c r="F7" s="14">
+        <v>2</v>
+      </c>
+      <c r="G7" s="14">
+        <v>11</v>
+      </c>
+      <c r="H7" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="N7" s="3"/>
+      <c r="O7" s="5"/>
+      <c r="P7" s="6"/>
+    </row>
+    <row r="8" spans="2:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="B8" s="19"/>
       <c r="C8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="19"/>
-      <c r="E8" s="19"/>
-      <c r="F8" s="19"/>
-      <c r="G8" s="19"/>
-      <c r="H8" s="16" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17">
+        <v>16</v>
+      </c>
+      <c r="H8" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="N8" s="3"/>
+      <c r="O8" s="5"/>
+      <c r="P8" s="6"/>
+    </row>
+    <row r="9" spans="2:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="N9" s="3"/>
+      <c r="O9" s="5"/>
+      <c r="P9" s="6"/>
+    </row>
+    <row r="10" spans="2:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="N10" s="3"/>
+      <c r="O10" s="5"/>
+      <c r="P10" s="6"/>
+    </row>
+    <row r="11" spans="2:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="N11" s="3"/>
+      <c r="O11" s="5"/>
+      <c r="P11" s="6"/>
+    </row>
+    <row r="12" spans="2:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="N12" s="3"/>
+      <c r="O12" s="5"/>
+      <c r="P12" s="6"/>
+    </row>
+    <row r="13" spans="2:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="N13" s="3"/>
+      <c r="O13" s="5"/>
+      <c r="P13" s="6"/>
+    </row>
+    <row r="14" spans="2:18" x14ac:dyDescent="0.55000000000000004">
       <c r="J14" s="3" t="s">
         <v>55</v>
       </c>
@@ -2106,8 +3330,20 @@
       <c r="L14" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="15" spans="2:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="M14" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="N14" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="O14" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="P14" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="2:18" x14ac:dyDescent="0.55000000000000004">
       <c r="J15" s="3">
         <v>1</v>
       </c>
@@ -2117,8 +3353,28 @@
       <c r="L15" s="6">
         <v>2</v>
       </c>
-    </row>
-    <row r="16" spans="2:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="M15" s="6">
+        <v>4</v>
+      </c>
+      <c r="N15" s="3">
+        <v>1</v>
+      </c>
+      <c r="O15" s="5">
+        <v>2</v>
+      </c>
+      <c r="P15" s="6">
+        <v>2</v>
+      </c>
+      <c r="Q15">
+        <f>P15*O15</f>
+        <v>4</v>
+      </c>
+      <c r="R15" t="str">
+        <f>IF(M15=Q15,"Gleich","Nicht Gleich")</f>
+        <v>Gleich</v>
+      </c>
+    </row>
+    <row r="16" spans="2:18" x14ac:dyDescent="0.55000000000000004">
       <c r="J16" s="3">
         <v>2</v>
       </c>
@@ -2128,8 +3384,28 @@
       <c r="L16" s="6">
         <v>3</v>
       </c>
-    </row>
-    <row r="17" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="M16" s="6">
+        <v>6</v>
+      </c>
+      <c r="N16" s="3">
+        <v>2</v>
+      </c>
+      <c r="O16" s="5">
+        <v>2</v>
+      </c>
+      <c r="P16" s="6">
+        <v>3</v>
+      </c>
+      <c r="Q16">
+        <f t="shared" ref="Q16:Q37" si="0">P16*O16</f>
+        <v>6</v>
+      </c>
+      <c r="R16" t="str">
+        <f t="shared" ref="R16:R37" si="1">IF(M16=Q16,"Gleich","Nicht Gleich")</f>
+        <v>Gleich</v>
+      </c>
+    </row>
+    <row r="17" spans="10:18" x14ac:dyDescent="0.55000000000000004">
       <c r="J17" s="3">
         <v>3</v>
       </c>
@@ -2139,19 +3415,59 @@
       <c r="L17" s="6">
         <v>2</v>
       </c>
-    </row>
-    <row r="18" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="J18" s="3">
-        <v>4</v>
-      </c>
-      <c r="K18" s="5">
-        <v>4</v>
-      </c>
-      <c r="L18" s="6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="M17" s="6">
+        <v>8</v>
+      </c>
+      <c r="N17" s="3">
+        <v>3</v>
+      </c>
+      <c r="O17" s="5">
+        <v>4</v>
+      </c>
+      <c r="P17" s="6">
+        <v>2</v>
+      </c>
+      <c r="Q17">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="R17" t="str">
+        <f t="shared" si="1"/>
+        <v>Gleich</v>
+      </c>
+    </row>
+    <row r="18" spans="10:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="J18" s="23">
+        <v>4</v>
+      </c>
+      <c r="K18" s="24">
+        <v>4</v>
+      </c>
+      <c r="L18" s="23">
+        <v>4</v>
+      </c>
+      <c r="M18" s="23">
+        <v>16</v>
+      </c>
+      <c r="N18" s="3">
+        <v>4</v>
+      </c>
+      <c r="O18" s="5">
+        <v>4</v>
+      </c>
+      <c r="P18" s="6">
+        <v>3</v>
+      </c>
+      <c r="Q18">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="R18" t="str">
+        <f t="shared" si="1"/>
+        <v>Nicht Gleich</v>
+      </c>
+    </row>
+    <row r="19" spans="10:18" x14ac:dyDescent="0.55000000000000004">
       <c r="J19" s="3">
         <v>5</v>
       </c>
@@ -2161,8 +3477,28 @@
       <c r="L19" s="6">
         <v>3</v>
       </c>
-    </row>
-    <row r="20" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="M19" s="6">
+        <v>9</v>
+      </c>
+      <c r="N19" s="3">
+        <v>5</v>
+      </c>
+      <c r="O19" s="5">
+        <v>3</v>
+      </c>
+      <c r="P19" s="6">
+        <v>3</v>
+      </c>
+      <c r="Q19">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="R19" t="str">
+        <f t="shared" si="1"/>
+        <v>Gleich</v>
+      </c>
+    </row>
+    <row r="20" spans="10:18" x14ac:dyDescent="0.55000000000000004">
       <c r="J20" s="3">
         <v>6</v>
       </c>
@@ -2172,8 +3508,28 @@
       <c r="L20" s="6">
         <v>3</v>
       </c>
-    </row>
-    <row r="21" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="M20" s="6">
+        <v>12</v>
+      </c>
+      <c r="N20" s="3">
+        <v>6</v>
+      </c>
+      <c r="O20" s="5">
+        <v>4</v>
+      </c>
+      <c r="P20" s="6">
+        <v>3</v>
+      </c>
+      <c r="Q20">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="R20" t="str">
+        <f t="shared" si="1"/>
+        <v>Gleich</v>
+      </c>
+    </row>
+    <row r="21" spans="10:18" x14ac:dyDescent="0.55000000000000004">
       <c r="J21" s="3">
         <v>7</v>
       </c>
@@ -2183,30 +3539,90 @@
       <c r="L21" s="6">
         <v>2</v>
       </c>
-    </row>
-    <row r="22" spans="10:12" x14ac:dyDescent="0.55000000000000004">
-      <c r="J22" s="3">
+      <c r="M21" s="6">
+        <v>6</v>
+      </c>
+      <c r="N21" s="3">
+        <v>7</v>
+      </c>
+      <c r="O21" s="5">
+        <v>3</v>
+      </c>
+      <c r="P21" s="6">
+        <v>2</v>
+      </c>
+      <c r="Q21">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="R21" t="str">
+        <f t="shared" si="1"/>
+        <v>Gleich</v>
+      </c>
+    </row>
+    <row r="22" spans="10:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="J22" s="23">
         <v>8</v>
       </c>
-      <c r="K22" s="5">
-        <v>5</v>
-      </c>
-      <c r="L22" s="6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="23" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="J23" s="3">
+      <c r="K22" s="24">
+        <v>5</v>
+      </c>
+      <c r="L22" s="23">
+        <v>4</v>
+      </c>
+      <c r="M22" s="23">
+        <v>20</v>
+      </c>
+      <c r="N22" s="3">
+        <v>8</v>
+      </c>
+      <c r="O22" s="5">
+        <v>4</v>
+      </c>
+      <c r="P22" s="6">
+        <v>4</v>
+      </c>
+      <c r="Q22">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="R22" t="str">
+        <f t="shared" si="1"/>
+        <v>Nicht Gleich</v>
+      </c>
+    </row>
+    <row r="23" spans="10:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="J23" s="23">
         <v>9</v>
       </c>
-      <c r="K23" s="5">
-        <v>3</v>
-      </c>
-      <c r="L23" s="6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="K23" s="27">
+        <v>3</v>
+      </c>
+      <c r="L23" s="28">
+        <v>3</v>
+      </c>
+      <c r="M23" s="28">
+        <v>9</v>
+      </c>
+      <c r="N23" s="3">
+        <v>9</v>
+      </c>
+      <c r="O23" s="5">
+        <v>3</v>
+      </c>
+      <c r="P23" s="6">
+        <v>4</v>
+      </c>
+      <c r="Q23">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="R23" t="str">
+        <f t="shared" si="1"/>
+        <v>Nicht Gleich</v>
+      </c>
+    </row>
+    <row r="24" spans="10:18" x14ac:dyDescent="0.55000000000000004">
       <c r="J24" s="3">
         <v>10</v>
       </c>
@@ -2216,118 +3632,338 @@
       <c r="L24" s="6">
         <v>3</v>
       </c>
-    </row>
-    <row r="25" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="J25" s="3">
+      <c r="M24" s="6">
+        <v>12</v>
+      </c>
+      <c r="N24" s="3">
+        <v>10</v>
+      </c>
+      <c r="O24" s="5">
+        <v>4</v>
+      </c>
+      <c r="P24" s="6">
+        <v>3</v>
+      </c>
+      <c r="Q24">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="R24" t="str">
+        <f t="shared" si="1"/>
+        <v>Gleich</v>
+      </c>
+    </row>
+    <row r="25" spans="10:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="J25" s="23">
         <v>11</v>
       </c>
-      <c r="K25" s="5">
-        <v>2</v>
-      </c>
-      <c r="L25" s="6">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="J26" s="3">
+      <c r="K25" s="24">
+        <v>2</v>
+      </c>
+      <c r="L25" s="23">
+        <v>4</v>
+      </c>
+      <c r="M25" s="23">
+        <v>8</v>
+      </c>
+      <c r="N25" s="3">
+        <v>11</v>
+      </c>
+      <c r="O25" s="5">
+        <v>2</v>
+      </c>
+      <c r="P25" s="6">
+        <v>5</v>
+      </c>
+      <c r="Q25">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="R25" t="str">
+        <f t="shared" si="1"/>
+        <v>Nicht Gleich</v>
+      </c>
+    </row>
+    <row r="26" spans="10:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="J26" s="23">
         <v>12</v>
       </c>
-      <c r="K26" s="5">
-        <v>4</v>
-      </c>
-      <c r="L26" s="6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="27" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="J27" s="3">
+      <c r="K26" s="24">
+        <v>4</v>
+      </c>
+      <c r="L26" s="23">
+        <v>4</v>
+      </c>
+      <c r="M26" s="23">
+        <v>16</v>
+      </c>
+      <c r="N26" s="3">
+        <v>12</v>
+      </c>
+      <c r="O26" s="5">
+        <v>4</v>
+      </c>
+      <c r="P26" s="6">
+        <v>3</v>
+      </c>
+      <c r="Q26">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="R26" t="str">
+        <f t="shared" si="1"/>
+        <v>Nicht Gleich</v>
+      </c>
+    </row>
+    <row r="27" spans="10:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="J27" s="23">
         <v>13</v>
       </c>
-      <c r="K27" s="5">
-        <v>2</v>
-      </c>
-      <c r="L27" s="6">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="28" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="K27" s="27">
+        <v>1</v>
+      </c>
+      <c r="L27" s="28">
+        <v>5</v>
+      </c>
+      <c r="M27" s="28">
+        <v>5</v>
+      </c>
+      <c r="N27" s="3">
+        <v>13</v>
+      </c>
+      <c r="O27" s="5">
+        <v>2</v>
+      </c>
+      <c r="P27" s="6">
+        <v>5</v>
+      </c>
+      <c r="Q27">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="R27" t="str">
+        <f t="shared" si="1"/>
+        <v>Nicht Gleich</v>
+      </c>
+    </row>
+    <row r="28" spans="10:18" x14ac:dyDescent="0.55000000000000004">
       <c r="J28" s="3">
         <v>14</v>
       </c>
       <c r="K28" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L28" s="6">
         <v>5</v>
       </c>
-    </row>
-    <row r="29" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="M28" s="6">
+        <v>10</v>
+      </c>
+      <c r="N28" s="3">
+        <v>14</v>
+      </c>
+      <c r="O28" s="5">
+        <v>2</v>
+      </c>
+      <c r="P28" s="6">
+        <v>5</v>
+      </c>
+      <c r="Q28">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="R28" t="str">
+        <f t="shared" si="1"/>
+        <v>Gleich</v>
+      </c>
+    </row>
+    <row r="29" spans="10:18" x14ac:dyDescent="0.55000000000000004">
       <c r="J29" s="3">
         <v>15</v>
       </c>
       <c r="K29" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L29" s="6">
         <v>5</v>
       </c>
-    </row>
-    <row r="30" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="J30" s="3">
+      <c r="M29" s="6">
+        <v>5</v>
+      </c>
+      <c r="N29" s="3">
+        <v>15</v>
+      </c>
+      <c r="O29" s="5">
+        <v>1</v>
+      </c>
+      <c r="P29" s="6">
+        <v>5</v>
+      </c>
+      <c r="Q29">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="R29" t="str">
+        <f t="shared" si="1"/>
+        <v>Gleich</v>
+      </c>
+    </row>
+    <row r="30" spans="10:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="J30" s="23">
         <v>16</v>
       </c>
-      <c r="K30" s="5">
+      <c r="K30" s="27">
         <v>1</v>
       </c>
-      <c r="L30" s="6">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="31" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="J31" s="3">
+      <c r="L30" s="28">
+        <v>4</v>
+      </c>
+      <c r="M30" s="28">
+        <v>4</v>
+      </c>
+      <c r="N30" s="3">
+        <v>16</v>
+      </c>
+      <c r="O30" s="5">
+        <v>2</v>
+      </c>
+      <c r="P30" s="6">
+        <v>4</v>
+      </c>
+      <c r="Q30">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="R30" t="str">
+        <f t="shared" si="1"/>
+        <v>Nicht Gleich</v>
+      </c>
+    </row>
+    <row r="31" spans="10:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="J31" s="23">
         <v>17</v>
       </c>
-      <c r="K31" s="5">
-        <v>2</v>
-      </c>
-      <c r="L31" s="6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="32" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="K31" s="24">
+        <v>3</v>
+      </c>
+      <c r="L31" s="23">
+        <v>5</v>
+      </c>
+      <c r="M31" s="23">
+        <v>15</v>
+      </c>
+      <c r="N31" s="3">
+        <v>17</v>
+      </c>
+      <c r="O31" s="5">
+        <v>1</v>
+      </c>
+      <c r="P31" s="6">
+        <v>5</v>
+      </c>
+      <c r="Q31">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="R31" t="str">
+        <f t="shared" si="1"/>
+        <v>Nicht Gleich</v>
+      </c>
+    </row>
+    <row r="32" spans="10:18" x14ac:dyDescent="0.55000000000000004">
       <c r="J32" s="3">
         <v>18</v>
       </c>
       <c r="K32" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L32" s="6">
         <v>5</v>
       </c>
-    </row>
-    <row r="33" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="M32" s="6">
+        <v>10</v>
+      </c>
+      <c r="N32" s="3">
+        <v>18</v>
+      </c>
+      <c r="O32" s="5">
+        <v>2</v>
+      </c>
+      <c r="P32" s="6">
+        <v>5</v>
+      </c>
+      <c r="Q32">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="R32" t="str">
+        <f t="shared" si="1"/>
+        <v>Gleich</v>
+      </c>
+    </row>
+    <row r="33" spans="10:18" x14ac:dyDescent="0.55000000000000004">
       <c r="J33" s="3">
         <v>19</v>
       </c>
       <c r="K33" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L33" s="6">
         <v>5</v>
       </c>
-    </row>
-    <row r="34" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="M33" s="6">
+        <v>5</v>
+      </c>
+      <c r="N33" s="3">
+        <v>19</v>
+      </c>
+      <c r="O33" s="5">
+        <v>1</v>
+      </c>
+      <c r="P33" s="6">
+        <v>5</v>
+      </c>
+      <c r="Q33">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="R33" t="str">
+        <f t="shared" si="1"/>
+        <v>Gleich</v>
+      </c>
+    </row>
+    <row r="34" spans="10:18" x14ac:dyDescent="0.55000000000000004">
       <c r="J34" s="3">
         <v>20</v>
       </c>
-      <c r="K34" s="5">
-        <v>1</v>
-      </c>
-      <c r="L34" s="6">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="35" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="K34" s="27">
+        <v>4</v>
+      </c>
+      <c r="L34" s="28">
+        <v>2</v>
+      </c>
+      <c r="M34" s="28">
+        <v>8</v>
+      </c>
+      <c r="N34" s="3">
+        <v>20</v>
+      </c>
+      <c r="O34" s="5">
+        <v>5</v>
+      </c>
+      <c r="P34" s="6">
+        <v>3</v>
+      </c>
+      <c r="Q34">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="R34" t="str">
+        <f t="shared" si="1"/>
+        <v>Nicht Gleich</v>
+      </c>
+    </row>
+    <row r="35" spans="10:18" x14ac:dyDescent="0.55000000000000004">
       <c r="J35" s="3">
         <v>21</v>
       </c>
@@ -2337,38 +3973,64 @@
       <c r="L35" s="6">
         <v>4</v>
       </c>
-    </row>
-    <row r="36" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="M35" s="6">
+        <v>12</v>
+      </c>
+      <c r="Q35">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R35" t="str">
+        <f t="shared" si="1"/>
+        <v>Nicht Gleich</v>
+      </c>
+    </row>
+    <row r="36" spans="10:18" x14ac:dyDescent="0.55000000000000004">
       <c r="J36" s="3">
         <v>22</v>
       </c>
       <c r="K36" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L36" s="6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="37" spans="10:12" hidden="1" x14ac:dyDescent="0.55000000000000004">
+        <v>4</v>
+      </c>
+      <c r="M36" s="6">
+        <v>12</v>
+      </c>
+      <c r="Q36">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R36" t="str">
+        <f t="shared" si="1"/>
+        <v>Nicht Gleich</v>
+      </c>
+    </row>
+    <row r="37" spans="10:18" x14ac:dyDescent="0.55000000000000004">
       <c r="J37" s="3">
         <v>23</v>
       </c>
       <c r="K37" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L37" s="6">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="M37" s="6">
+        <v>5</v>
+      </c>
+      <c r="Q37">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R37" t="str">
+        <f t="shared" si="1"/>
+        <v>Nicht Gleich</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="J1:L37" xr:uid="{38F3AE2C-2824-4C08-B947-28E1493E0DC2}">
-    <filterColumn colId="1">
-      <filters blank="1">
-        <filter val="5"/>
-        <filter val="Likelyhood"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="J1:L37" xr:uid="{38F3AE2C-2824-4C08-B947-28E1493E0DC2}"/>
   <mergeCells count="2">
     <mergeCell ref="D2:H2"/>
     <mergeCell ref="B2:B8"/>
@@ -2377,7 +4039,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D11458A-F0B2-4399-BAB5-99C5BA883F62}">
   <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
@@ -2720,7 +4382,7 @@
         <v>52</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D20" s="5">
         <v>2</v>
@@ -2734,7 +4396,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B24E2C4B-86F0-456F-9E76-A960D71BEE17}">
   <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
@@ -2757,10 +4419,10 @@
         <v>25</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>84</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
@@ -2811,7 +4473,7 @@
         <v>59</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
@@ -2887,7 +4549,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>29</v>
@@ -2904,7 +4566,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>31</v>
@@ -3070,10 +4732,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>59</v>
@@ -3087,7 +4749,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{037AD151-7D7B-4E13-A86C-35CB016C1B9B}">
   <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
@@ -3106,10 +4768,10 @@
         <v>0</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
@@ -3120,7 +4782,7 @@
         <v>19</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D2" s="8">
         <v>72981</v>
@@ -3134,7 +4796,7 @@
         <v>21</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D3" s="6"/>
     </row>
@@ -3146,7 +4808,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D4" s="8">
         <v>45953</v>
@@ -3160,7 +4822,7 @@
         <v>17</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D5" s="8">
         <v>45953</v>
@@ -3174,7 +4836,7 @@
         <v>75</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D6" s="8">
         <v>45953</v>
@@ -3188,7 +4850,7 @@
         <v>79</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D7" s="8">
         <v>45940</v>
@@ -3202,7 +4864,7 @@
         <v>24</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D8" s="8">
         <v>45947</v>
@@ -3216,7 +4878,7 @@
         <v>28</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D9" s="8">
         <v>45953</v>
@@ -3230,7 +4892,7 @@
         <v>30</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D10" s="8">
         <v>45953</v>
@@ -3244,7 +4906,7 @@
         <v>33</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D11" s="8">
         <v>45953</v>
@@ -3258,10 +4920,10 @@
         <v>35</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
@@ -3272,7 +4934,7 @@
         <v>38</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D13" s="8">
         <v>45953</v>
@@ -3286,7 +4948,7 @@
         <v>40</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D14" s="8">
         <v>45940</v>
@@ -3300,7 +4962,7 @@
         <v>43</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D15" s="8">
         <v>45947</v>
@@ -3314,7 +4976,7 @@
         <v>45</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D16" s="8">
         <v>45940</v>
@@ -3328,7 +4990,7 @@
         <v>48</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D17" s="8">
         <v>45926</v>
@@ -3342,7 +5004,7 @@
         <v>50</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D18" s="8">
         <v>45926</v>
@@ -3356,7 +5018,7 @@
         <v>53</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D19" s="8">
         <v>45953</v>
@@ -3367,10 +5029,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D20" s="8">
         <v>45953</v>
@@ -3381,7 +5043,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A62239C4-D2DC-4635-A96D-B4AE35CFCD8F}">
   <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
@@ -3402,19 +5064,19 @@
         <v>0</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E1" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="F1" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="F1" s="9" t="s">
-        <v>109</v>
-      </c>
       <c r="G1" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -3425,11 +5087,11 @@
         <v>19</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D2" s="6"/>
       <c r="E2" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -3440,11 +5102,11 @@
         <v>21</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -3455,16 +5117,16 @@
         <v>1</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E4" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="F4" t="s">
         <v>125</v>
-      </c>
-      <c r="F4" t="s">
-        <v>126</v>
       </c>
       <c r="G4" s="10">
         <v>46227</v>
@@ -3478,16 +5140,16 @@
         <v>17</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D5" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="E5" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="F5" t="s">
         <v>132</v>
-      </c>
-      <c r="F5" t="s">
-        <v>133</v>
       </c>
       <c r="G5" s="10">
         <v>46227</v>
@@ -3501,13 +5163,13 @@
         <v>75</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D6" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="E6" s="8" t="s">
         <v>123</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>124</v>
       </c>
       <c r="G6" s="10">
         <v>46227</v>
@@ -3521,13 +5183,13 @@
         <v>79</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D7" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="E7" s="8" t="s">
         <v>121</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>122</v>
       </c>
       <c r="G7" s="10"/>
     </row>
@@ -3539,14 +5201,14 @@
         <v>24</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G8" s="10">
         <v>46227</v>
@@ -3560,7 +5222,7 @@
         <v>28</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="8"/>
@@ -3573,7 +5235,7 @@
         <v>30</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="8"/>
@@ -3586,7 +5248,7 @@
         <v>33</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="8"/>
@@ -3599,7 +5261,7 @@
         <v>35</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
@@ -3612,7 +5274,7 @@
         <v>38</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="8"/>
@@ -3625,7 +5287,7 @@
         <v>40</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="8"/>
@@ -3638,7 +5300,7 @@
         <v>43</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="8"/>
@@ -3651,7 +5313,7 @@
         <v>45</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="8"/>
@@ -3664,7 +5326,7 @@
         <v>48</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="8"/>
@@ -3677,7 +5339,7 @@
         <v>50</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="8"/>
@@ -3690,7 +5352,7 @@
         <v>53</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D19" s="6"/>
       <c r="E19" s="8"/>
@@ -3700,10 +5362,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D20" s="6"/>
       <c r="E20" s="8"/>
@@ -3713,19 +5375,19 @@
         <v>20</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D21" t="s">
+        <v>127</v>
+      </c>
+      <c r="E21" t="s">
         <v>128</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>129</v>
-      </c>
-      <c r="F21" t="s">
-        <v>130</v>
       </c>
       <c r="G21" s="10">
         <v>46204</v>

</xml_diff>

<commit_message>
first version with project management closed
</commit_message>
<xml_diff>
--- a/content/tables/Risk_Mgmt.xlsx
+++ b/content/tables/Risk_Mgmt.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BFH\MSE\MSE_MasterThesis\content\tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBDF98A1-9C73-4045-98A2-EEEDBA3AC342}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA470192-3953-4FB2-9F3D-00253666FB71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{C85C79CF-50DE-474C-BA2B-673335091AFF}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" activeTab="3" xr2:uid="{C85C79CF-50DE-474C-BA2B-673335091AFF}"/>
   </bookViews>
   <sheets>
     <sheet name="Table with Risks and Measures" sheetId="5" r:id="rId1"/>
     <sheet name="Table with Risks_Projekt2" sheetId="13" r:id="rId2"/>
     <sheet name="Graphical Overview" sheetId="4" r:id="rId3"/>
-    <sheet name="RiskEval" sheetId="6" r:id="rId4"/>
-    <sheet name="RiskTreatment" sheetId="7" r:id="rId5"/>
-    <sheet name="RiskWhatWhen" sheetId="8" r:id="rId6"/>
-    <sheet name="CheckinOct" sheetId="12" r:id="rId7"/>
+    <sheet name="Graphical Overview (2)" sheetId="14" r:id="rId4"/>
+    <sheet name="RiskEval" sheetId="6" r:id="rId5"/>
+    <sheet name="RiskTreatment" sheetId="7" r:id="rId6"/>
+    <sheet name="RiskWhatWhen" sheetId="8" r:id="rId7"/>
+    <sheet name="CheckinOct" sheetId="12" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Graphical Overview'!$J$1:$L$37</definedName>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="185">
   <si>
     <t>Risk</t>
   </si>
@@ -297,6 +298,9 @@
     <t>To be documented in miro calendar case it happens</t>
   </si>
   <si>
+    <t>4, 6, 10, 12</t>
+  </si>
+  <si>
     <t>Treatment</t>
   </si>
   <si>
@@ -486,9 +490,6 @@
     <t>Providing continous feedback and having weekly call are done to find missing contributions early</t>
   </si>
   <si>
-    <t>Reduce: Part of Jour Fixe</t>
-  </si>
-  <si>
     <t>Setup calls early, search external resources always before starting work blocks</t>
   </si>
   <si>
@@ -553,6 +554,54 @@
   </si>
   <si>
     <t>The required management process is unknown</t>
+  </si>
+  <si>
+    <t>Reduce: In the research section smart goals have been setup</t>
+  </si>
+  <si>
+    <t>Reduce: The introduction describes which parts of the initial project description are part of this document</t>
+  </si>
+  <si>
+    <t>Reduce: Phases and Milestones are set up as progress checks</t>
+  </si>
+  <si>
+    <t>Reduce: Discussed availability with other team, added blockers in work calendar, work account invited to meeting Series (Jour Fixe), study Account: Set blockers on weekend, researched with ChatGPT for optimal or minimal study plan</t>
+  </si>
+  <si>
+    <t>Reduce: Work on he project started 14.09.2026, first meeting with expert in same week</t>
+  </si>
+  <si>
+    <t>Reduce: Contact of partner provided in teams, and added to Miro board</t>
+  </si>
+  <si>
+    <t>Transfer: Asked for contact, confirmed to be Jürgen Vogel</t>
+  </si>
+  <si>
+    <t>Second Laptop is available at home, The Latex document is a Github project, documentation is on miro. Work laptop can also be used for most tasks, but has no Latex installed</t>
+  </si>
+  <si>
+    <t>Reduce: Github project for Latex document</t>
+  </si>
+  <si>
+    <t>Reduce: Jabref used as GUI for biblliography, Biber used for build</t>
+  </si>
+  <si>
+    <t>Reduce: Jour fixe setup</t>
+  </si>
+  <si>
+    <t>Reduce: Keep exchange chanells also when changing team</t>
+  </si>
+  <si>
+    <t>Reduce: Part of Jour fixe</t>
+  </si>
+  <si>
+    <t>2, 7</t>
+  </si>
+  <si>
+    <t>11, 14</t>
+  </si>
+  <si>
+    <t>15, 17, 19</t>
   </si>
 </sst>
 </file>
@@ -641,12 +690,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.89999084444715716"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -654,6 +697,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -696,7 +745,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
@@ -730,20 +779,26 @@
       <alignment horizontal="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1078,23 +1133,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01ACE7B3-DC9E-49CA-A001-535C01F14776}">
-  <dimension ref="A1:X33"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.89453125" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="10.89453125" style="2"/>
-    <col min="2" max="2" width="26.7890625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="50.20703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="25.5234375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.1015625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.26171875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="21" width="10.89453125" style="1"/>
-    <col min="22" max="22" width="51.47265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="14.15625" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="16384" width="10.89453125" style="1"/>
+    <col min="1" max="1" width="10.89453125" style="3"/>
+    <col min="2" max="2" width="26.7890625" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50.20703125" style="6" customWidth="1"/>
+    <col min="4" max="4" width="25.5234375" style="6" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="9.1015625" style="6" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="6.734375" style="6" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="20.26171875" style="6" hidden="1" customWidth="1"/>
+    <col min="8" max="11" width="10.89453125" style="6"/>
+    <col min="12" max="12" width="86" style="6" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="146.3671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="10.89453125" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="23.7" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:14" ht="23.7" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="3" t="s">
         <v>55</v>
       </c>
@@ -1128,41 +1184,17 @@
       <c r="K1" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="L1" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="M1" s="20" t="s">
-        <v>4</v>
-      </c>
-      <c r="N1" s="20" t="s">
-        <v>56</v>
-      </c>
-      <c r="O1" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="P1" s="21" t="s">
-        <v>77</v>
-      </c>
-      <c r="Q1" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="R1" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="S1" s="3"/>
-      <c r="T1" s="3"/>
-      <c r="U1" s="3"/>
-      <c r="V1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="M1" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="N1" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="X1" s="3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="2" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="2" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -1185,36 +1217,20 @@
         <f>E2*F2</f>
         <v>4</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="L2" s="22">
-        <v>2</v>
-      </c>
-      <c r="M2" s="20">
-        <v>2</v>
-      </c>
-      <c r="N2" s="20">
-        <f>L2*M2</f>
-        <v>4</v>
-      </c>
-      <c r="O2" s="21"/>
-      <c r="P2" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q2" s="21"/>
-      <c r="R2" s="21"/>
-      <c r="V2" s="1" t="s">
+      <c r="L2" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="W2" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="X2" s="7">
+      <c r="M2" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="N2" s="8">
         <v>46319</v>
       </c>
     </row>
-    <row r="3" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -1237,36 +1253,20 @@
         <f t="shared" ref="G3:G23" si="0">E3*F3</f>
         <v>6</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="L3" s="22">
-        <v>2</v>
-      </c>
-      <c r="M3" s="20">
-        <v>3</v>
-      </c>
-      <c r="N3" s="20">
-        <f>L3*M3</f>
-        <v>6</v>
-      </c>
-      <c r="O3" s="21"/>
-      <c r="P3" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q3" s="21"/>
-      <c r="R3" s="21"/>
-      <c r="V3" s="1" t="s">
+      <c r="L3" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="W3" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="X3" s="7">
+      <c r="M3" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="N3" s="8">
         <v>46319</v>
       </c>
     </row>
-    <row r="4" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -1289,85 +1289,56 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="H4" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="L4" s="22">
-        <v>4</v>
-      </c>
-      <c r="M4" s="20">
-        <v>2</v>
-      </c>
-      <c r="N4" s="20">
-        <f>L4*M4</f>
-        <v>8</v>
-      </c>
-      <c r="O4" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="P4" s="21"/>
-      <c r="Q4" s="21"/>
-      <c r="R4" s="21"/>
-      <c r="V4" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="W4" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="X4" s="7">
+      <c r="L4" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="N4" s="8">
         <v>46319</v>
       </c>
     </row>
-    <row r="5" spans="1:24" s="25" customFormat="1" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="23">
-        <v>4</v>
-      </c>
-      <c r="B5" s="23" t="s">
+    <row r="5" spans="1:14" s="20" customFormat="1" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="20">
+        <v>4</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="C5" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="D5" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="24">
-        <v>4</v>
-      </c>
-      <c r="F5" s="23">
-        <v>4</v>
-      </c>
-      <c r="G5" s="23">
+      <c r="E5" s="21">
+        <v>4</v>
+      </c>
+      <c r="F5" s="20">
+        <v>4</v>
+      </c>
+      <c r="G5" s="20">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="I5" s="25" t="s">
+      <c r="I5" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="L5" s="24">
-        <v>4</v>
-      </c>
-      <c r="M5" s="23">
-        <v>3</v>
-      </c>
-      <c r="N5" s="23">
-        <f>L5*M5</f>
-        <v>12</v>
-      </c>
-      <c r="O5" s="25" t="s">
-        <v>57</v>
-      </c>
-      <c r="V5" s="25" t="s">
-        <v>143</v>
-      </c>
-      <c r="W5" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="X5" s="26">
+      <c r="L5" s="20" t="s">
+        <v>144</v>
+      </c>
+      <c r="M5" s="20" t="s">
+        <v>171</v>
+      </c>
+      <c r="N5" s="24">
         <v>46319</v>
       </c>
     </row>
-    <row r="6" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -1390,36 +1361,20 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="L6" s="22">
-        <v>3</v>
-      </c>
-      <c r="M6" s="20">
-        <v>3</v>
-      </c>
-      <c r="N6" s="20">
-        <f>L6*M6</f>
-        <v>9</v>
-      </c>
-      <c r="O6" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="P6" s="21"/>
-      <c r="Q6" s="21"/>
-      <c r="R6" s="21"/>
-      <c r="V6" s="1" t="s">
+      <c r="L6" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="W6" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="X6" s="7">
+      <c r="M6" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="N6" s="8">
         <v>46319</v>
       </c>
     </row>
-    <row r="7" spans="1:24" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:14" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -1442,36 +1397,20 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="I7" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="L7" s="22">
-        <v>4</v>
-      </c>
-      <c r="M7" s="20">
-        <v>3</v>
-      </c>
-      <c r="N7" s="20">
-        <f>L7*M7</f>
-        <v>12</v>
-      </c>
-      <c r="O7" s="21"/>
-      <c r="P7" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q7" s="21"/>
-      <c r="R7" s="21"/>
-      <c r="V7" s="1" t="s">
+      <c r="L7" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="W7" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="X7" s="7">
+      <c r="M7" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="N7" s="8">
         <v>46319</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -1494,134 +1433,92 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="I8" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="L8" s="22">
-        <v>3</v>
-      </c>
-      <c r="M8" s="20">
-        <v>2</v>
-      </c>
-      <c r="N8" s="20">
-        <f>L8*M8</f>
-        <v>6</v>
-      </c>
-      <c r="O8" s="21"/>
-      <c r="P8" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q8" s="21"/>
-      <c r="R8" s="21"/>
-      <c r="V8" s="1" t="s">
+      <c r="L8" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="W8" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="X8" s="7">
+      <c r="M8" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="N8" s="8">
         <v>46319</v>
       </c>
     </row>
-    <row r="9" spans="1:24" s="25" customFormat="1" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="23">
+    <row r="9" spans="1:14" s="20" customFormat="1" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="20">
         <v>8</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="24" t="s">
+      <c r="D9" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="E9" s="24">
-        <v>5</v>
-      </c>
-      <c r="F9" s="23">
-        <v>4</v>
-      </c>
-      <c r="G9" s="23">
+      <c r="E9" s="21">
+        <v>5</v>
+      </c>
+      <c r="F9" s="20">
+        <v>4</v>
+      </c>
+      <c r="G9" s="20">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="I9" s="25" t="s">
+      <c r="I9" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="L9" s="24">
-        <v>4</v>
-      </c>
-      <c r="M9" s="23">
-        <v>4</v>
-      </c>
-      <c r="N9" s="23">
-        <f>L9*M9</f>
-        <v>16</v>
-      </c>
-      <c r="P9" s="25" t="s">
-        <v>57</v>
-      </c>
-      <c r="V9" s="25" t="s">
-        <v>144</v>
-      </c>
-      <c r="W9" s="25" t="s">
-        <v>93</v>
-      </c>
-      <c r="X9" s="26">
+      <c r="L9" s="20" t="s">
+        <v>145</v>
+      </c>
+      <c r="M9" s="20" t="s">
+        <v>174</v>
+      </c>
+      <c r="N9" s="24">
         <v>46319</v>
       </c>
     </row>
-    <row r="10" spans="1:24" s="25" customFormat="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="23">
+    <row r="10" spans="1:14" s="20" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="20">
         <v>9</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="C10" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="24" t="s">
+      <c r="D10" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="E10" s="27">
-        <v>3</v>
-      </c>
-      <c r="F10" s="28">
-        <v>3</v>
-      </c>
-      <c r="G10" s="28">
+      <c r="E10" s="22">
+        <v>3</v>
+      </c>
+      <c r="F10" s="23">
+        <v>3</v>
+      </c>
+      <c r="G10" s="23">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="J10" s="25" t="s">
+      <c r="J10" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="L10" s="24">
-        <v>3</v>
-      </c>
-      <c r="M10" s="23">
-        <v>4</v>
-      </c>
-      <c r="N10" s="23">
-        <f>L10*M10</f>
-        <v>12</v>
-      </c>
-      <c r="Q10" s="25" t="s">
-        <v>57</v>
-      </c>
-      <c r="V10" s="25" t="s">
+      <c r="L10" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="W10" s="25" t="s">
-        <v>94</v>
-      </c>
-      <c r="X10" s="26">
+      <c r="M10" s="20" t="s">
+        <v>175</v>
+      </c>
+      <c r="N10" s="24">
         <v>46319</v>
       </c>
     </row>
-    <row r="11" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -1644,183 +1541,128 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="H11" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="L11" s="22">
-        <v>4</v>
-      </c>
-      <c r="M11" s="20">
-        <v>3</v>
-      </c>
-      <c r="N11" s="20">
-        <f>L11*M11</f>
-        <v>12</v>
-      </c>
-      <c r="O11" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="P11" s="21"/>
-      <c r="Q11" s="21"/>
-      <c r="R11" s="21"/>
-      <c r="V11" s="1" t="s">
+      <c r="L11" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="W11" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="X11" s="7">
+      <c r="M11" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="N11" s="8">
         <v>46319</v>
       </c>
     </row>
-    <row r="12" spans="1:24" s="25" customFormat="1" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="23">
+    <row r="12" spans="1:14" s="20" customFormat="1" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="20">
         <v>11</v>
       </c>
-      <c r="B12" s="23" t="s">
+      <c r="B12" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="24" t="s">
+      <c r="C12" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="24" t="s">
+      <c r="D12" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="E12" s="24">
-        <v>2</v>
-      </c>
-      <c r="F12" s="23">
-        <v>4</v>
-      </c>
-      <c r="G12" s="23">
+      <c r="E12" s="21">
+        <v>2</v>
+      </c>
+      <c r="F12" s="20">
+        <v>4</v>
+      </c>
+      <c r="G12" s="20">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="I12" s="25" t="s">
+      <c r="I12" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="L12" s="24">
-        <v>2</v>
-      </c>
-      <c r="M12" s="23">
-        <v>5</v>
-      </c>
-      <c r="N12" s="23">
-        <f>L12*M12</f>
-        <v>10</v>
-      </c>
-      <c r="P12" s="25" t="s">
-        <v>57</v>
-      </c>
-      <c r="V12" s="25" t="s">
+      <c r="L12" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="W12" s="25" t="s">
-        <v>96</v>
-      </c>
-      <c r="X12" s="26">
+      <c r="M12" s="20" t="s">
+        <v>176</v>
+      </c>
+      <c r="N12" s="24">
         <v>46319</v>
       </c>
     </row>
-    <row r="13" spans="1:24" s="25" customFormat="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="23">
+    <row r="13" spans="1:14" s="20" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="20">
         <v>12</v>
       </c>
-      <c r="B13" s="23" t="s">
+      <c r="B13" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="24" t="s">
+      <c r="C13" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="D13" s="24" t="s">
+      <c r="D13" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="E13" s="24">
-        <v>4</v>
-      </c>
-      <c r="F13" s="23">
-        <v>4</v>
-      </c>
-      <c r="G13" s="23">
+      <c r="E13" s="21">
+        <v>4</v>
+      </c>
+      <c r="F13" s="20">
+        <v>4</v>
+      </c>
+      <c r="G13" s="20">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="H13" s="25" t="s">
+      <c r="H13" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="L13" s="24">
-        <v>4</v>
-      </c>
-      <c r="M13" s="23">
-        <v>3</v>
-      </c>
-      <c r="N13" s="23">
-        <f>L13*M13</f>
-        <v>12</v>
-      </c>
-      <c r="O13" s="25" t="s">
+      <c r="L13" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="M13" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="N13" s="24">
+        <v>46319</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" s="20" customFormat="1" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="20">
+        <v>13</v>
+      </c>
+      <c r="B14" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="E14" s="22">
+        <v>1</v>
+      </c>
+      <c r="F14" s="23">
+        <v>5</v>
+      </c>
+      <c r="G14" s="23">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="I14" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="V13" s="25" t="s">
-        <v>97</v>
-      </c>
-      <c r="W13" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="X13" s="26">
+      <c r="L14" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="M14" s="20" t="s">
+        <v>177</v>
+      </c>
+      <c r="N14" s="24">
         <v>46319</v>
       </c>
     </row>
-    <row r="14" spans="1:24" s="25" customFormat="1" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="23">
-        <v>13</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="D14" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="E14" s="27">
-        <v>1</v>
-      </c>
-      <c r="F14" s="28">
-        <v>5</v>
-      </c>
-      <c r="G14" s="28">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="I14" s="25" t="s">
-        <v>57</v>
-      </c>
-      <c r="L14" s="24">
-        <v>2</v>
-      </c>
-      <c r="M14" s="23">
-        <v>5</v>
-      </c>
-      <c r="N14" s="23">
-        <f>L14*M14</f>
-        <v>10</v>
-      </c>
-      <c r="P14" s="25" t="s">
-        <v>57</v>
-      </c>
-      <c r="V14" s="25" t="s">
-        <v>98</v>
-      </c>
-      <c r="W14" s="25" t="s">
-        <v>99</v>
-      </c>
-      <c r="X14" s="26">
-        <v>46319</v>
-      </c>
-    </row>
-    <row r="15" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -1843,36 +1685,20 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="I15" s="1" t="s">
+      <c r="I15" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="L15" s="22">
-        <v>2</v>
-      </c>
-      <c r="M15" s="20">
-        <v>5</v>
-      </c>
-      <c r="N15" s="20">
-        <f>L15*M15</f>
-        <v>10</v>
-      </c>
-      <c r="O15" s="21"/>
-      <c r="P15" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q15" s="21"/>
-      <c r="R15" s="21"/>
-      <c r="V15" s="1" t="s">
+      <c r="L15" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="W15" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="X15" s="7">
+      <c r="M15" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="N15" s="8">
         <v>46319</v>
       </c>
     </row>
-    <row r="16" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -1895,134 +1721,92 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="H16" s="1" t="s">
+      <c r="H16" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="L16" s="22">
+      <c r="L16" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="M16" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="N16" s="8">
+        <v>46319</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" s="20" customFormat="1" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17" s="20">
+        <v>16</v>
+      </c>
+      <c r="B17" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="E17" s="22">
         <v>1</v>
       </c>
-      <c r="M16" s="20">
-        <v>5</v>
-      </c>
-      <c r="N16" s="20">
-        <f>L16*M16</f>
-        <v>5</v>
-      </c>
-      <c r="O16" s="21" t="s">
+      <c r="F17" s="23">
+        <v>4</v>
+      </c>
+      <c r="G17" s="23">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="I17" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="P16" s="21"/>
-      <c r="Q16" s="21"/>
-      <c r="R16" s="21"/>
-      <c r="V16" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="W16" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="X16" s="7">
+      <c r="L17" s="20" t="s">
+        <v>103</v>
+      </c>
+      <c r="M17" s="20" t="s">
+        <v>179</v>
+      </c>
+      <c r="N17" s="24">
         <v>46319</v>
       </c>
     </row>
-    <row r="17" spans="1:24" s="25" customFormat="1" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A17" s="23">
-        <v>16</v>
-      </c>
-      <c r="B17" s="23" t="s">
+    <row r="18" spans="1:14" s="20" customFormat="1" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" s="20">
+        <v>17</v>
+      </c>
+      <c r="B18" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="D17" s="24" t="s">
-        <v>49</v>
-      </c>
-      <c r="E17" s="27">
-        <v>1</v>
-      </c>
-      <c r="F17" s="28">
-        <v>4</v>
-      </c>
-      <c r="G17" s="28">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="I17" s="25" t="s">
-        <v>57</v>
-      </c>
-      <c r="L17" s="24">
-        <v>2</v>
-      </c>
-      <c r="M17" s="23">
-        <v>4</v>
-      </c>
-      <c r="N17" s="23">
-        <f>L17*M17</f>
-        <v>8</v>
-      </c>
-      <c r="P17" s="25" t="s">
-        <v>57</v>
-      </c>
-      <c r="V17" s="25" t="s">
-        <v>102</v>
-      </c>
-      <c r="W17" s="25" t="s">
-        <v>103</v>
-      </c>
-      <c r="X17" s="26">
-        <v>46319</v>
-      </c>
-    </row>
-    <row r="18" spans="1:24" s="25" customFormat="1" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" s="23">
-        <v>17</v>
-      </c>
-      <c r="B18" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="C18" s="24" t="s">
+      <c r="C18" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="D18" s="24" t="s">
+      <c r="D18" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="E18" s="24">
-        <v>3</v>
-      </c>
-      <c r="F18" s="23">
-        <v>5</v>
-      </c>
-      <c r="G18" s="23">
+      <c r="E18" s="21">
+        <v>3</v>
+      </c>
+      <c r="F18" s="20">
+        <v>5</v>
+      </c>
+      <c r="G18" s="20">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="I18" s="25" t="s">
+      <c r="I18" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="L18" s="24">
-        <v>1</v>
-      </c>
-      <c r="M18" s="23">
-        <v>5</v>
-      </c>
-      <c r="N18" s="23">
-        <f>L18*M18</f>
-        <v>5</v>
-      </c>
-      <c r="P18" s="25" t="s">
-        <v>57</v>
-      </c>
-      <c r="V18" s="25" t="s">
+      <c r="L18" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="W18" s="25" t="s">
-        <v>104</v>
-      </c>
-      <c r="X18" s="26">
+      <c r="M18" s="20" t="s">
+        <v>180</v>
+      </c>
+      <c r="N18" s="24">
         <v>46319</v>
       </c>
     </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -2045,36 +1829,20 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="H19" s="1" t="s">
+      <c r="H19" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="L19" s="22">
-        <v>2</v>
-      </c>
-      <c r="M19" s="20">
-        <v>5</v>
-      </c>
-      <c r="N19" s="20">
-        <f>L19*M19</f>
-        <v>10</v>
-      </c>
-      <c r="O19" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="P19" s="21"/>
-      <c r="Q19" s="21"/>
-      <c r="R19" s="21"/>
-      <c r="V19" s="1" t="s">
+      <c r="L19" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="W19" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="X19" s="7">
+      <c r="M19" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="N19" s="8">
         <v>46319</v>
       </c>
     </row>
-    <row r="20" spans="1:24" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:14" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -2082,10 +1850,10 @@
         <v>52</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E20" s="5">
         <v>1</v>
@@ -2097,41 +1865,25 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="H20" s="1" t="s">
+      <c r="H20" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="L20" s="22">
-        <v>1</v>
-      </c>
-      <c r="M20" s="20">
-        <v>5</v>
-      </c>
-      <c r="N20" s="20">
-        <f>L20*M20</f>
-        <v>5</v>
-      </c>
-      <c r="O20" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="P20" s="21"/>
-      <c r="Q20" s="21"/>
-      <c r="R20" s="21"/>
-      <c r="V20" s="1" t="s">
+      <c r="L20" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="W20" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="X20" s="7">
+      <c r="M20" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="N20" s="8">
         <v>46319</v>
       </c>
     </row>
-    <row r="21" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="3">
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>168</v>
@@ -2139,46 +1891,30 @@
       <c r="D21" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="E21" s="27">
-        <v>4</v>
-      </c>
-      <c r="F21" s="28">
-        <v>2</v>
-      </c>
-      <c r="G21" s="28">
+      <c r="E21" s="22">
+        <v>4</v>
+      </c>
+      <c r="F21" s="23">
+        <v>2</v>
+      </c>
+      <c r="G21" s="23">
         <f>E21*F21</f>
         <v>8</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="I21" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="L21" s="22">
-        <v>5</v>
-      </c>
-      <c r="M21" s="20">
-        <v>3</v>
-      </c>
-      <c r="N21" s="20">
-        <f>L21*M21</f>
-        <v>15</v>
-      </c>
-      <c r="O21" s="21"/>
-      <c r="P21" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q21" s="21"/>
-      <c r="R21" s="21"/>
-      <c r="V21" s="1" t="s">
+      <c r="L21" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="W21" s="1" t="s">
+      <c r="M21" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="X21" s="7">
+      <c r="N21" s="8">
         <v>46319</v>
       </c>
     </row>
-    <row r="22" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -2186,10 +1922,10 @@
         <v>47</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E22" s="5">
         <v>3</v>
@@ -2201,31 +1937,31 @@
         <f>E22*F22</f>
         <v>12</v>
       </c>
-      <c r="I22" s="1" t="s">
+      <c r="I22" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="V22" s="1" t="s">
+      <c r="L22" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="W22" s="1" t="s">
+      <c r="M22" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="X22" s="7">
+      <c r="N22" s="8">
         <v>46319</v>
       </c>
     </row>
-    <row r="23" spans="1:24" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:14" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="3">
         <v>22</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C23" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="D23" s="5" t="s">
         <v>140</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>139</v>
       </c>
       <c r="E23" s="5">
         <v>3</v>
@@ -2237,20 +1973,20 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="H23" s="1" t="s">
+      <c r="H23" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="V23" s="1" t="s">
+      <c r="L23" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="W23" s="1" t="s">
+      <c r="M23" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="X23" s="7">
+      <c r="N23" s="8">
         <v>46319</v>
       </c>
     </row>
-    <row r="24" spans="1:24" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:14" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -2258,7 +1994,7 @@
         <v>37</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>166</v>
@@ -2273,73 +2009,61 @@
         <f>E24*F24</f>
         <v>5</v>
       </c>
-      <c r="I24" s="1" t="s">
+      <c r="I24" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="V24" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="W24" s="1" t="s">
+      <c r="L24" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="X24" s="7">
+      <c r="M24" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="N24" s="8">
         <v>46319</v>
       </c>
     </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.55000000000000004">
-      <c r="A25" s="3"/>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="B25" s="3"/>
       <c r="C25" s="5"/>
       <c r="D25" s="5"/>
       <c r="E25" s="5"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-      <c r="X25" s="7"/>
-    </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="3"/>
+      <c r="N25" s="8"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="B26" s="3"/>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
       <c r="E26" s="5"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="X26" s="7"/>
-    </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.55000000000000004">
-      <c r="A27" s="3"/>
+      <c r="N26" s="8"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="B27" s="3"/>
-      <c r="C27"/>
+      <c r="C27" s="25"/>
       <c r="D27" s="5"/>
       <c r="E27" s="5"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
-      <c r="X27" s="7"/>
-    </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.55000000000000004">
-      <c r="A28" s="3"/>
+      <c r="N27" s="8"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="B28" s="3"/>
-      <c r="C28"/>
+      <c r="C28" s="25"/>
       <c r="D28" s="5"/>
       <c r="E28" s="5"/>
-      <c r="F28" s="6"/>
-      <c r="G28" s="6"/>
-      <c r="X28" s="7"/>
-    </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.55000000000000004">
-      <c r="C29"/>
-    </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.55000000000000004">
-      <c r="C30"/>
-    </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.55000000000000004">
-      <c r="C31"/>
-    </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.55000000000000004">
-      <c r="C32"/>
+      <c r="N28" s="8"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="C29" s="25"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="C30" s="25"/>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="C31" s="25"/>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="C32" s="25"/>
     </row>
     <row r="33" spans="3:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="C33"/>
+      <c r="C33" s="25"/>
     </row>
   </sheetData>
   <autoFilter ref="E1:E33" xr:uid="{01ACE7B3-DC9E-49CA-A001-535C01F14776}"/>
@@ -2403,10 +2127,10 @@
         <v>62</v>
       </c>
       <c r="V1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="W1" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>88</v>
       </c>
       <c r="X1" s="1" t="s">
         <v>158</v>
@@ -2445,7 +2169,7 @@
         <v>71</v>
       </c>
       <c r="V2" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="W2" s="7">
         <v>72981</v>
@@ -2481,7 +2205,7 @@
         <v>72</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:25" ht="28.8" x14ac:dyDescent="0.55000000000000004">
@@ -2514,7 +2238,7 @@
         <v>156</v>
       </c>
       <c r="V4" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="W4" s="7">
         <v>45953</v>
@@ -2550,7 +2274,7 @@
         <v>70</v>
       </c>
       <c r="V5" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="W5" s="7">
         <v>45953</v>
@@ -2586,7 +2310,7 @@
         <v>78</v>
       </c>
       <c r="V6" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="W6" s="7">
         <v>45953</v>
@@ -2622,7 +2346,7 @@
         <v>81</v>
       </c>
       <c r="V7" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="W7" s="7">
         <v>45940</v>
@@ -2658,7 +2382,7 @@
         <v>63</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="W8" s="7">
         <v>45947</v>
@@ -2694,7 +2418,7 @@
         <v>155</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="W9" s="7">
         <v>45953</v>
@@ -2730,7 +2454,7 @@
         <v>68</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="W10" s="7">
         <v>45953</v>
@@ -2766,7 +2490,7 @@
         <v>73</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="W11" s="7">
         <v>45953</v>
@@ -2802,10 +2526,10 @@
         <v>67</v>
       </c>
       <c r="V12" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="W12" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="W12" s="1" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.55000000000000004">
@@ -2835,10 +2559,10 @@
         <v>57</v>
       </c>
       <c r="U13" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="V13" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="W13" s="7">
         <v>45953</v>
@@ -2871,10 +2595,10 @@
         <v>57</v>
       </c>
       <c r="U14" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="V14" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="W14" s="7">
         <v>45940</v>
@@ -2910,7 +2634,7 @@
         <v>65</v>
       </c>
       <c r="V15" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="W15" s="7">
         <v>45947</v>
@@ -2943,10 +2667,10 @@
         <v>57</v>
       </c>
       <c r="U16" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="V16" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="W16" s="7">
         <v>45940</v>
@@ -2979,10 +2703,10 @@
         <v>57</v>
       </c>
       <c r="U17" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="V17" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="W17" s="7">
         <v>45926</v>
@@ -3018,7 +2742,7 @@
         <v>74</v>
       </c>
       <c r="V18" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="W18" s="7">
         <v>45926</v>
@@ -3054,7 +2778,7 @@
         <v>82</v>
       </c>
       <c r="V19" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="W19" s="7">
         <v>45953</v>
@@ -3068,10 +2792,10 @@
         <v>52</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E20" s="5">
         <v>1</v>
@@ -3090,7 +2814,7 @@
         <v>82</v>
       </c>
       <c r="V20" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="W20" s="7">
         <v>45953</v>
@@ -3101,13 +2825,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E21" s="5">
         <v>5</v>
@@ -3282,7 +3006,7 @@
       <c r="C8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="17"/>
+      <c r="D8" s="30"/>
       <c r="E8" s="17"/>
       <c r="F8" s="17"/>
       <c r="G8" s="17">
@@ -3437,16 +3161,16 @@
       </c>
     </row>
     <row r="18" spans="10:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="J18" s="23">
-        <v>4</v>
-      </c>
-      <c r="K18" s="24">
-        <v>4</v>
-      </c>
-      <c r="L18" s="23">
-        <v>4</v>
-      </c>
-      <c r="M18" s="23">
+      <c r="J18" s="20">
+        <v>4</v>
+      </c>
+      <c r="K18" s="21">
+        <v>4</v>
+      </c>
+      <c r="L18" s="20">
+        <v>4</v>
+      </c>
+      <c r="M18" s="20">
         <v>16</v>
       </c>
       <c r="N18" s="3">
@@ -3561,16 +3285,16 @@
       </c>
     </row>
     <row r="22" spans="10:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="J22" s="23">
+      <c r="J22" s="20">
         <v>8</v>
       </c>
-      <c r="K22" s="24">
-        <v>5</v>
-      </c>
-      <c r="L22" s="23">
-        <v>4</v>
-      </c>
-      <c r="M22" s="23">
+      <c r="K22" s="21">
+        <v>5</v>
+      </c>
+      <c r="L22" s="20">
+        <v>4</v>
+      </c>
+      <c r="M22" s="20">
         <v>20</v>
       </c>
       <c r="N22" s="3">
@@ -3592,16 +3316,16 @@
       </c>
     </row>
     <row r="23" spans="10:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="J23" s="23">
+      <c r="J23" s="20">
         <v>9</v>
       </c>
-      <c r="K23" s="27">
-        <v>3</v>
-      </c>
-      <c r="L23" s="28">
-        <v>3</v>
-      </c>
-      <c r="M23" s="28">
+      <c r="K23" s="22">
+        <v>3</v>
+      </c>
+      <c r="L23" s="23">
+        <v>3</v>
+      </c>
+      <c r="M23" s="23">
         <v>9</v>
       </c>
       <c r="N23" s="3">
@@ -3654,16 +3378,16 @@
       </c>
     </row>
     <row r="25" spans="10:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="J25" s="23">
+      <c r="J25" s="20">
         <v>11</v>
       </c>
-      <c r="K25" s="24">
-        <v>2</v>
-      </c>
-      <c r="L25" s="23">
-        <v>4</v>
-      </c>
-      <c r="M25" s="23">
+      <c r="K25" s="21">
+        <v>2</v>
+      </c>
+      <c r="L25" s="20">
+        <v>4</v>
+      </c>
+      <c r="M25" s="20">
         <v>8</v>
       </c>
       <c r="N25" s="3">
@@ -3685,16 +3409,16 @@
       </c>
     </row>
     <row r="26" spans="10:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="J26" s="23">
+      <c r="J26" s="20">
         <v>12</v>
       </c>
-      <c r="K26" s="24">
-        <v>4</v>
-      </c>
-      <c r="L26" s="23">
-        <v>4</v>
-      </c>
-      <c r="M26" s="23">
+      <c r="K26" s="21">
+        <v>4</v>
+      </c>
+      <c r="L26" s="20">
+        <v>4</v>
+      </c>
+      <c r="M26" s="20">
         <v>16</v>
       </c>
       <c r="N26" s="3">
@@ -3716,16 +3440,16 @@
       </c>
     </row>
     <row r="27" spans="10:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="J27" s="23">
+      <c r="J27" s="20">
         <v>13</v>
       </c>
-      <c r="K27" s="27">
+      <c r="K27" s="22">
         <v>1</v>
       </c>
-      <c r="L27" s="28">
-        <v>5</v>
-      </c>
-      <c r="M27" s="28">
+      <c r="L27" s="23">
+        <v>5</v>
+      </c>
+      <c r="M27" s="23">
         <v>5</v>
       </c>
       <c r="N27" s="3">
@@ -3809,16 +3533,16 @@
       </c>
     </row>
     <row r="30" spans="10:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="J30" s="23">
+      <c r="J30" s="20">
         <v>16</v>
       </c>
-      <c r="K30" s="27">
+      <c r="K30" s="22">
         <v>1</v>
       </c>
-      <c r="L30" s="28">
-        <v>4</v>
-      </c>
-      <c r="M30" s="28">
+      <c r="L30" s="23">
+        <v>4</v>
+      </c>
+      <c r="M30" s="23">
         <v>4</v>
       </c>
       <c r="N30" s="3">
@@ -3840,16 +3564,16 @@
       </c>
     </row>
     <row r="31" spans="10:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="J31" s="23">
+      <c r="J31" s="20">
         <v>17</v>
       </c>
-      <c r="K31" s="24">
-        <v>3</v>
-      </c>
-      <c r="L31" s="23">
-        <v>5</v>
-      </c>
-      <c r="M31" s="23">
+      <c r="K31" s="21">
+        <v>3</v>
+      </c>
+      <c r="L31" s="20">
+        <v>5</v>
+      </c>
+      <c r="M31" s="20">
         <v>15</v>
       </c>
       <c r="N31" s="3">
@@ -3936,13 +3660,13 @@
       <c r="J34" s="3">
         <v>20</v>
       </c>
-      <c r="K34" s="27">
-        <v>4</v>
-      </c>
-      <c r="L34" s="28">
-        <v>2</v>
-      </c>
-      <c r="M34" s="28">
+      <c r="K34" s="22">
+        <v>4</v>
+      </c>
+      <c r="L34" s="23">
+        <v>2</v>
+      </c>
+      <c r="M34" s="23">
         <v>8</v>
       </c>
       <c r="N34" s="3">
@@ -4036,10 +3760,396 @@
     <mergeCell ref="B2:B8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="E5" twoDigitTextYear="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9CB0573-9312-435B-A218-8989D53C9D2B}">
+  <dimension ref="B1:M22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="3" max="3" width="12.15625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.9453125" style="2"/>
+    <col min="11" max="11" width="9.1015625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.734375" style="1" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="J1" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="2:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="B2" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="28" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="J2" s="3">
+        <v>1</v>
+      </c>
+      <c r="K2" s="5">
+        <v>2</v>
+      </c>
+      <c r="L2" s="6">
+        <v>2</v>
+      </c>
+      <c r="M2" s="26"/>
+    </row>
+    <row r="3" spans="2:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="B3" s="27"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" s="3">
+        <v>2</v>
+      </c>
+      <c r="K3" s="5">
+        <v>2</v>
+      </c>
+      <c r="L3" s="6">
+        <v>3</v>
+      </c>
+      <c r="M3" s="26"/>
+    </row>
+    <row r="4" spans="2:13" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B4" s="27"/>
+      <c r="C4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+      <c r="J4" s="3">
+        <v>3</v>
+      </c>
+      <c r="K4" s="5">
+        <v>4</v>
+      </c>
+      <c r="L4" s="6">
+        <v>2</v>
+      </c>
+      <c r="M4" s="26"/>
+    </row>
+    <row r="5" spans="2:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="B5" s="27"/>
+      <c r="C5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="14">
+        <v>21</v>
+      </c>
+      <c r="E5" s="15">
+        <v>16</v>
+      </c>
+      <c r="F5" s="15">
+        <v>9</v>
+      </c>
+      <c r="G5" s="16">
+        <v>8</v>
+      </c>
+      <c r="H5" s="16"/>
+      <c r="J5" s="3">
+        <v>4</v>
+      </c>
+      <c r="K5" s="5">
+        <v>4</v>
+      </c>
+      <c r="L5" s="6">
+        <v>3</v>
+      </c>
+      <c r="M5" s="26"/>
+    </row>
+    <row r="6" spans="2:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="B6" s="27"/>
+      <c r="C6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="17"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="15">
+        <v>5</v>
+      </c>
+      <c r="G6" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="H6" s="16"/>
+      <c r="J6" s="3">
+        <v>5</v>
+      </c>
+      <c r="K6" s="5">
+        <v>3</v>
+      </c>
+      <c r="L6" s="6">
+        <v>3</v>
+      </c>
+      <c r="M6" s="26"/>
+    </row>
+    <row r="7" spans="2:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="B7" s="27"/>
+      <c r="C7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17">
+        <v>1</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="G7" s="14">
+        <v>3</v>
+      </c>
+      <c r="H7" s="15"/>
+      <c r="J7" s="3">
+        <v>6</v>
+      </c>
+      <c r="K7" s="5">
+        <v>4</v>
+      </c>
+      <c r="L7" s="6">
+        <v>3</v>
+      </c>
+      <c r="M7" s="26"/>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="B8" s="27"/>
+      <c r="C8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="14"/>
+      <c r="J8" s="3">
+        <v>7</v>
+      </c>
+      <c r="K8" s="5">
+        <v>3</v>
+      </c>
+      <c r="L8" s="6">
+        <v>2</v>
+      </c>
+      <c r="M8" s="26"/>
+    </row>
+    <row r="9" spans="2:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="J9" s="3">
+        <v>8</v>
+      </c>
+      <c r="K9" s="5">
+        <v>4</v>
+      </c>
+      <c r="L9" s="6">
+        <v>4</v>
+      </c>
+      <c r="M9" s="26"/>
+    </row>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="J10" s="3">
+        <v>9</v>
+      </c>
+      <c r="K10" s="5">
+        <v>3</v>
+      </c>
+      <c r="L10" s="6">
+        <v>4</v>
+      </c>
+      <c r="M10" s="26"/>
+    </row>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="J11" s="3">
+        <v>10</v>
+      </c>
+      <c r="K11" s="5">
+        <v>4</v>
+      </c>
+      <c r="L11" s="6">
+        <v>3</v>
+      </c>
+      <c r="M11" s="26"/>
+    </row>
+    <row r="12" spans="2:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="J12" s="3">
+        <v>11</v>
+      </c>
+      <c r="K12" s="5">
+        <v>2</v>
+      </c>
+      <c r="L12" s="6">
+        <v>5</v>
+      </c>
+      <c r="M12" s="26"/>
+    </row>
+    <row r="13" spans="2:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="J13" s="3">
+        <v>12</v>
+      </c>
+      <c r="K13" s="5">
+        <v>4</v>
+      </c>
+      <c r="L13" s="6">
+        <v>3</v>
+      </c>
+      <c r="M13" s="26"/>
+    </row>
+    <row r="14" spans="2:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="J14" s="3">
+        <v>13</v>
+      </c>
+      <c r="K14" s="5">
+        <v>2</v>
+      </c>
+      <c r="L14" s="6">
+        <v>5</v>
+      </c>
+      <c r="M14" s="26"/>
+    </row>
+    <row r="15" spans="2:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="J15" s="3">
+        <v>14</v>
+      </c>
+      <c r="K15" s="5">
+        <v>2</v>
+      </c>
+      <c r="L15" s="6">
+        <v>5</v>
+      </c>
+      <c r="M15" s="26"/>
+    </row>
+    <row r="16" spans="2:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="J16" s="3">
+        <v>15</v>
+      </c>
+      <c r="K16" s="5">
+        <v>1</v>
+      </c>
+      <c r="L16" s="6">
+        <v>5</v>
+      </c>
+      <c r="M16" s="26"/>
+    </row>
+    <row r="17" spans="10:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="J17" s="3">
+        <v>16</v>
+      </c>
+      <c r="K17" s="5">
+        <v>2</v>
+      </c>
+      <c r="L17" s="6">
+        <v>4</v>
+      </c>
+      <c r="M17" s="26"/>
+    </row>
+    <row r="18" spans="10:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="J18" s="3">
+        <v>17</v>
+      </c>
+      <c r="K18" s="5">
+        <v>1</v>
+      </c>
+      <c r="L18" s="6">
+        <v>5</v>
+      </c>
+      <c r="M18" s="26"/>
+    </row>
+    <row r="19" spans="10:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="J19" s="3">
+        <v>18</v>
+      </c>
+      <c r="K19" s="5">
+        <v>2</v>
+      </c>
+      <c r="L19" s="6">
+        <v>5</v>
+      </c>
+      <c r="M19" s="26"/>
+    </row>
+    <row r="20" spans="10:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="J20" s="3">
+        <v>19</v>
+      </c>
+      <c r="K20" s="5">
+        <v>2</v>
+      </c>
+      <c r="L20" s="6">
+        <v>5</v>
+      </c>
+      <c r="M20" s="26"/>
+    </row>
+    <row r="21" spans="10:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="J21" s="3">
+        <v>20</v>
+      </c>
+      <c r="K21" s="5">
+        <v>1</v>
+      </c>
+      <c r="L21" s="6">
+        <v>5</v>
+      </c>
+      <c r="M21" s="26"/>
+    </row>
+    <row r="22" spans="10:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="J22" s="3">
+        <v>21</v>
+      </c>
+      <c r="K22" s="5">
+        <v>1</v>
+      </c>
+      <c r="L22" s="6">
+        <v>4</v>
+      </c>
+      <c r="M22" s="26"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="B2:B8"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="E4" twoDigitTextYear="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D11458A-F0B2-4399-BAB5-99C5BA883F62}">
   <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
@@ -4382,7 +4492,7 @@
         <v>52</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D20" s="5">
         <v>2</v>
@@ -4396,7 +4506,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B24E2C4B-86F0-456F-9E76-A960D71BEE17}">
   <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
@@ -4419,10 +4529,10 @@
         <v>25</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
@@ -4473,7 +4583,7 @@
         <v>59</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
@@ -4549,7 +4659,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>29</v>
@@ -4566,7 +4676,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>31</v>
@@ -4732,10 +4842,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>116</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>115</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>59</v>
@@ -4749,7 +4859,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{037AD151-7D7B-4E13-A86C-35CB016C1B9B}">
   <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
@@ -4768,10 +4878,10 @@
         <v>0</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>89</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
@@ -4782,7 +4892,7 @@
         <v>19</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D2" s="8">
         <v>72981</v>
@@ -4796,7 +4906,7 @@
         <v>21</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D3" s="6"/>
     </row>
@@ -4808,7 +4918,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D4" s="8">
         <v>45953</v>
@@ -4822,7 +4932,7 @@
         <v>17</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D5" s="8">
         <v>45953</v>
@@ -4836,7 +4946,7 @@
         <v>75</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D6" s="8">
         <v>45953</v>
@@ -4850,7 +4960,7 @@
         <v>79</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D7" s="8">
         <v>45940</v>
@@ -4864,7 +4974,7 @@
         <v>24</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D8" s="8">
         <v>45947</v>
@@ -4878,7 +4988,7 @@
         <v>28</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D9" s="8">
         <v>45953</v>
@@ -4892,7 +5002,7 @@
         <v>30</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D10" s="8">
         <v>45953</v>
@@ -4906,7 +5016,7 @@
         <v>33</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D11" s="8">
         <v>45953</v>
@@ -4920,10 +5030,10 @@
         <v>35</v>
       </c>
       <c r="C12" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D12" s="6" t="s">
         <v>96</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
@@ -4934,7 +5044,7 @@
         <v>38</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D13" s="8">
         <v>45953</v>
@@ -4948,7 +5058,7 @@
         <v>40</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D14" s="8">
         <v>45940</v>
@@ -4962,7 +5072,7 @@
         <v>43</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D15" s="8">
         <v>45947</v>
@@ -4976,7 +5086,7 @@
         <v>45</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D16" s="8">
         <v>45940</v>
@@ -4990,7 +5100,7 @@
         <v>48</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D17" s="8">
         <v>45926</v>
@@ -5004,7 +5114,7 @@
         <v>50</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D18" s="8">
         <v>45926</v>
@@ -5018,7 +5128,7 @@
         <v>53</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D19" s="8">
         <v>45953</v>
@@ -5029,10 +5139,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D20" s="8">
         <v>45953</v>
@@ -5043,7 +5153,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A62239C4-D2DC-4635-A96D-B4AE35CFCD8F}">
   <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
@@ -5064,19 +5174,19 @@
         <v>0</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="E1" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="F1" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="E1" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>108</v>
-      </c>
       <c r="G1" s="9" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -5087,11 +5197,11 @@
         <v>19</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D2" s="6"/>
       <c r="E2" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -5102,11 +5212,11 @@
         <v>21</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="8" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -5117,16 +5227,16 @@
         <v>1</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G4" s="10">
         <v>46227</v>
@@ -5140,16 +5250,16 @@
         <v>17</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G5" s="10">
         <v>46227</v>
@@ -5163,13 +5273,13 @@
         <v>75</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G6" s="10">
         <v>46227</v>
@@ -5183,13 +5293,13 @@
         <v>79</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G7" s="10"/>
     </row>
@@ -5201,14 +5311,14 @@
         <v>24</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G8" s="10">
         <v>46227</v>
@@ -5222,7 +5332,7 @@
         <v>28</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="8"/>
@@ -5235,7 +5345,7 @@
         <v>30</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="8"/>
@@ -5248,7 +5358,7 @@
         <v>33</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="8"/>
@@ -5261,7 +5371,7 @@
         <v>35</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
@@ -5274,7 +5384,7 @@
         <v>38</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="8"/>
@@ -5287,7 +5397,7 @@
         <v>40</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="8"/>
@@ -5300,7 +5410,7 @@
         <v>43</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="8"/>
@@ -5313,7 +5423,7 @@
         <v>45</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="8"/>
@@ -5326,7 +5436,7 @@
         <v>48</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="8"/>
@@ -5339,7 +5449,7 @@
         <v>50</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="8"/>
@@ -5352,7 +5462,7 @@
         <v>53</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D19" s="6"/>
       <c r="E19" s="8"/>
@@ -5362,10 +5472,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D20" s="6"/>
       <c r="E20" s="8"/>
@@ -5375,19 +5485,19 @@
         <v>20</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D21" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E21" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F21" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G21" s="10">
         <v>46204</v>

</xml_diff>